<commit_message>
tn to kg measure update added in export contract
</commit_message>
<xml_diff>
--- a/templates/Export_Agreement.xlsx
+++ b/templates/Export_Agreement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\papka\TSAddIn\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tsAddin\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81A8488-1D39-4C17-8275-0379DD0D10B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5428E2-66C5-4818-8E14-35FF8B822CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1837" yWindow="4230" windowWidth="21600" windowHeight="11423" activeTab="1" xr2:uid="{B6FC3AD6-F63C-4057-BD0B-525C27FA51AB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6FC3AD6-F63C-4057-BD0B-525C27FA51AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Export_Contract" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,6 @@
     <definedName name="Invoice_sign_seller_start">Invoice!$J$41</definedName>
     <definedName name="MID_Contract">Export_Contract!$E$1</definedName>
     <definedName name="MID_Invoice">Invoice!$G$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Invoice!$A$1:$N$50</definedName>
     <definedName name="Seal_agent_end">Export_Contract!$H$66</definedName>
     <definedName name="Seal_agent_start">Export_Contract!$G$56</definedName>
     <definedName name="Seal_seller_end">Export_Contract!$C$66</definedName>
@@ -83,6 +82,7 @@
     <definedName name="Контракт">Export_Contract!$B$3</definedName>
     <definedName name="Контракт_дата">Export_Contract!$B$4</definedName>
     <definedName name="Контракт_предмет_заголовки">Export_Contract!$B$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Invoice!$A$1:$N$50</definedName>
     <definedName name="Остальное_контракт">Export_Contract!$B$29</definedName>
     <definedName name="Покупатель">Export_Contract!$B$12</definedName>
     <definedName name="Покупатель_адрес">Export_Contract!$B$13</definedName>
@@ -244,14 +244,6 @@
     <t>Продавец обязуется поставить Покупателю, а Покупатель обязуется принять и оплатить партию следующей продукции:</t>
   </si>
   <si>
-    <t xml:space="preserve">Цена, $/тн  
-Price, $/tn </t>
-  </si>
-  <si>
-    <t>Кол-во, тн 
-Quantity, tn</t>
-  </si>
-  <si>
     <t>A/C: 40702840201401167199</t>
   </si>
   <si>
@@ -290,14 +282,6 @@
 Сумма, $</t>
   </si>
   <si>
-    <t>Price, $/тн
-Цена, $/tn</t>
-  </si>
-  <si>
-    <t>Quantity, tn
-Количество, тн</t>
-  </si>
-  <si>
     <t>PCS /
 Места /</t>
   </si>
@@ -498,6 +482,22 @@
   </si>
   <si>
     <t>A/C:</t>
+  </si>
+  <si>
+    <t>Quantity, kg
+Количество, кг</t>
+  </si>
+  <si>
+    <t>Price, $/кг
+Цена, $/kg</t>
+  </si>
+  <si>
+    <t>Цена, $/кг
+Price, $/kg</t>
+  </si>
+  <si>
+    <t>Кол-во, кг
+Quantity, kg</t>
   </si>
 </sst>
 </file>
@@ -1344,6 +1344,81 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1362,81 +1437,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1451,8 +1451,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent 2" xfId="1" xr:uid="{5CD1A812-51BC-4B98-9C17-9ADDF6D1B6E6}"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1513,7 +1513,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office 2013–2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1831,43 +1831,43 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF102"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.06640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" style="41" customWidth="1"/>
-    <col min="3" max="3" width="23.59765625" style="41" customWidth="1"/>
+    <col min="1" max="1" width="1" style="7" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="41" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" style="41" customWidth="1"/>
     <col min="4" max="4" width="18" style="41" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" style="41" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="41" customWidth="1"/>
-    <col min="7" max="7" width="21.53125" style="41" customWidth="1"/>
-    <col min="8" max="8" width="12.265625" style="41" customWidth="1"/>
-    <col min="9" max="9" width="15.06640625" style="41" customWidth="1"/>
-    <col min="10" max="10" width="1.06640625" style="41" customWidth="1"/>
-    <col min="11" max="11" width="8.796875" style="7"/>
+    <col min="5" max="5" width="11.7109375" style="41" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" style="41" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" style="41" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="41" customWidth="1"/>
+    <col min="9" max="9" width="15" style="41" customWidth="1"/>
+    <col min="10" max="10" width="1" style="41" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" style="7"/>
     <col min="12" max="12" width="13" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.796875" style="7"/>
-    <col min="14" max="14" width="17.6640625" style="9" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" style="7"/>
+    <col min="14" max="14" width="17.7109375" style="9" customWidth="1"/>
     <col min="15" max="15" width="9" style="9" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="16.33203125" style="9" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="20.33203125" style="9" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="9.33203125" style="9" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="15.796875" style="9" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="49.796875" style="9" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="10.6640625" style="9" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="13.796875" style="9" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="7.33203125" style="9" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="9.796875" style="9" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="23.33203125" style="9" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="16.28515625" style="9" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="20.28515625" style="9" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="9.28515625" style="9" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="15.85546875" style="9" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="49.85546875" style="9" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="10.7109375" style="9" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="13.85546875" style="9" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="7.28515625" style="9" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="9.85546875" style="9" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="23.28515625" style="9" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="0" style="9" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="17.6640625" style="9" customWidth="1"/>
-    <col min="28" max="28" width="13.1328125" style="9" customWidth="1"/>
-    <col min="29" max="29" width="9.06640625" style="9" customWidth="1"/>
-    <col min="30" max="30" width="35.3984375" style="9" customWidth="1"/>
-    <col min="31" max="32" width="9.1328125" style="7" hidden="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.796875" style="7"/>
+    <col min="27" max="27" width="17.7109375" style="9" customWidth="1"/>
+    <col min="28" max="28" width="13.140625" style="9" customWidth="1"/>
+    <col min="29" max="29" width="9" style="9" customWidth="1"/>
+    <col min="30" max="30" width="35.42578125" style="9" customWidth="1"/>
+    <col min="31" max="32" width="9.140625" style="7" hidden="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.85546875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" ht="2.75" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:30" ht="2.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="143"/>
       <c r="C1" s="143"/>
       <c r="D1" s="143"/>
@@ -1879,19 +1879,19 @@
       <c r="H1" s="143"/>
       <c r="I1" s="143"/>
     </row>
-    <row r="2" spans="2:30" s="14" customFormat="1" ht="21.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="197" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="198"/>
-      <c r="D2" s="198"/>
-      <c r="E2" s="199"/>
-      <c r="F2" s="197" t="s">
-        <v>88</v>
-      </c>
-      <c r="G2" s="198"/>
-      <c r="H2" s="198"/>
-      <c r="I2" s="198"/>
+    <row r="2" spans="2:30" s="14" customFormat="1" ht="21.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="222" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="223"/>
+      <c r="D2" s="223"/>
+      <c r="E2" s="224"/>
+      <c r="F2" s="222" t="s">
+        <v>84</v>
+      </c>
+      <c r="G2" s="223"/>
+      <c r="H2" s="223"/>
+      <c r="I2" s="223"/>
       <c r="J2" s="144"/>
       <c r="L2" s="8"/>
       <c r="N2" s="15"/>
@@ -1900,19 +1900,19 @@
       <c r="AC2" s="15"/>
       <c r="AD2" s="15"/>
     </row>
-    <row r="3" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="200" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="201"/>
-      <c r="D3" s="201"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="200" t="s">
-        <v>89</v>
-      </c>
-      <c r="G3" s="201"/>
-      <c r="H3" s="201"/>
-      <c r="I3" s="201"/>
+    <row r="3" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="225" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="226"/>
+      <c r="D3" s="226"/>
+      <c r="E3" s="227"/>
+      <c r="F3" s="225" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="226"/>
+      <c r="H3" s="226"/>
+      <c r="I3" s="226"/>
       <c r="J3" s="6"/>
       <c r="L3" s="8"/>
       <c r="O3" s="7"/>
@@ -1928,19 +1928,19 @@
       <c r="Y3" s="7"/>
       <c r="Z3" s="7"/>
     </row>
-    <row r="4" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="200" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="201"/>
-      <c r="D4" s="201"/>
-      <c r="E4" s="202"/>
-      <c r="F4" s="200" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="201"/>
-      <c r="H4" s="201"/>
-      <c r="I4" s="201"/>
+    <row r="4" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="225" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="226"/>
+      <c r="D4" s="226"/>
+      <c r="E4" s="227"/>
+      <c r="F4" s="225" t="s">
+        <v>86</v>
+      </c>
+      <c r="G4" s="226"/>
+      <c r="H4" s="226"/>
+      <c r="I4" s="226"/>
       <c r="J4" s="6"/>
       <c r="N4" s="10"/>
       <c r="O4" s="11"/>
@@ -1960,19 +1960,19 @@
       <c r="AC4" s="10"/>
       <c r="AD4" s="10"/>
     </row>
-    <row r="5" spans="2:30" s="14" customFormat="1" ht="13.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="206" t="s">
+    <row r="5" spans="2:30" s="14" customFormat="1" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="218" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="207"/>
-      <c r="D5" s="207"/>
-      <c r="E5" s="208"/>
-      <c r="F5" s="206" t="s">
+      <c r="C5" s="219"/>
+      <c r="D5" s="219"/>
+      <c r="E5" s="220"/>
+      <c r="F5" s="218" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="207"/>
-      <c r="H5" s="207"/>
-      <c r="I5" s="207"/>
+      <c r="G5" s="219"/>
+      <c r="H5" s="219"/>
+      <c r="I5" s="219"/>
       <c r="J5" s="13"/>
       <c r="N5" s="15"/>
       <c r="AA5" s="15"/>
@@ -1980,7 +1980,7 @@
       <c r="AC5" s="15"/>
       <c r="AD5" s="15"/>
     </row>
-    <row r="6" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="161" t="s">
         <v>22</v>
       </c>
@@ -2008,15 +2008,15 @@
       <c r="Y6" s="7"/>
       <c r="Z6" s="7"/>
     </row>
-    <row r="7" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="161" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C7" s="164"/>
       <c r="D7" s="164"/>
       <c r="E7" s="165"/>
       <c r="F7" s="161" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G7" s="164"/>
       <c r="H7" s="164"/>
@@ -2036,45 +2036,45 @@
       <c r="Y7" s="7"/>
       <c r="Z7" s="7"/>
     </row>
-    <row r="8" spans="2:30" ht="13.15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="209" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" s="210"/>
-      <c r="D8" s="210"/>
-      <c r="E8" s="211"/>
-      <c r="F8" s="209" t="s">
-        <v>94</v>
-      </c>
-      <c r="G8" s="210"/>
-      <c r="H8" s="210"/>
-      <c r="I8" s="210"/>
+    <row r="8" spans="2:30" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="207" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="208"/>
+      <c r="D8" s="208"/>
+      <c r="E8" s="221"/>
+      <c r="F8" s="207" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="208"/>
+      <c r="H8" s="208"/>
+      <c r="I8" s="208"/>
       <c r="J8" s="19"/>
     </row>
-    <row r="9" spans="2:30" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="203" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" s="204"/>
-      <c r="D9" s="204"/>
-      <c r="E9" s="205"/>
-      <c r="F9" s="203" t="s">
-        <v>96</v>
-      </c>
-      <c r="G9" s="204"/>
-      <c r="H9" s="204"/>
-      <c r="I9" s="205"/>
+    <row r="9" spans="2:30" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="197" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="198"/>
+      <c r="D9" s="198"/>
+      <c r="E9" s="199"/>
+      <c r="F9" s="197" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="198"/>
+      <c r="H9" s="198"/>
+      <c r="I9" s="199"/>
       <c r="J9" s="19"/>
     </row>
-    <row r="10" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="203"/>
-      <c r="C10" s="204"/>
-      <c r="D10" s="204"/>
-      <c r="E10" s="205"/>
-      <c r="F10" s="203"/>
-      <c r="G10" s="204"/>
-      <c r="H10" s="204"/>
-      <c r="I10" s="205"/>
+    <row r="10" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="197"/>
+      <c r="C10" s="198"/>
+      <c r="D10" s="198"/>
+      <c r="E10" s="199"/>
+      <c r="F10" s="197"/>
+      <c r="G10" s="198"/>
+      <c r="H10" s="198"/>
+      <c r="I10" s="199"/>
       <c r="J10" s="19"/>
       <c r="N10" s="15"/>
       <c r="O10" s="7"/>
@@ -2094,7 +2094,7 @@
       <c r="AC10" s="15"/>
       <c r="AD10" s="15"/>
     </row>
-    <row r="11" spans="2:30" ht="16.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:30" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="158" t="s">
         <v>25</v>
       </c>
@@ -2121,15 +2121,15 @@
       <c r="Y11" s="7"/>
       <c r="Z11" s="7"/>
     </row>
-    <row r="12" spans="2:30" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:30" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="161" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="157"/>
       <c r="F12" s="161" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="164"/>
@@ -2148,19 +2148,19 @@
       <c r="Y12" s="7"/>
       <c r="Z12" s="7"/>
     </row>
-    <row r="13" spans="2:30" ht="27.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="203" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" s="204"/>
-      <c r="D13" s="204"/>
-      <c r="E13" s="205"/>
-      <c r="F13" s="203" t="s">
-        <v>98</v>
-      </c>
-      <c r="G13" s="204"/>
-      <c r="H13" s="204"/>
-      <c r="I13" s="204"/>
+    <row r="13" spans="2:30" ht="27.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="197" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13" s="198"/>
+      <c r="D13" s="198"/>
+      <c r="E13" s="199"/>
+      <c r="F13" s="197" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" s="198"/>
+      <c r="H13" s="198"/>
+      <c r="I13" s="198"/>
       <c r="J13" s="19"/>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
@@ -2177,19 +2177,19 @@
       <c r="Z13" s="7"/>
       <c r="AA13" s="7"/>
     </row>
-    <row r="14" spans="2:30" ht="13.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="203" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" s="204"/>
-      <c r="D14" s="204"/>
-      <c r="E14" s="205"/>
-      <c r="F14" s="203" t="s">
-        <v>100</v>
-      </c>
-      <c r="G14" s="204"/>
-      <c r="H14" s="204"/>
-      <c r="I14" s="204"/>
+    <row r="14" spans="2:30" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="197" t="s">
+        <v>95</v>
+      </c>
+      <c r="C14" s="198"/>
+      <c r="D14" s="198"/>
+      <c r="E14" s="199"/>
+      <c r="F14" s="197" t="s">
+        <v>96</v>
+      </c>
+      <c r="G14" s="198"/>
+      <c r="H14" s="198"/>
+      <c r="I14" s="198"/>
       <c r="J14" s="19"/>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
@@ -2206,19 +2206,19 @@
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
     </row>
-    <row r="15" spans="2:30" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="203" t="s">
+    <row r="15" spans="2:30" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="197" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="204"/>
-      <c r="D15" s="204"/>
-      <c r="E15" s="205"/>
-      <c r="F15" s="203" t="s">
+      <c r="C15" s="198"/>
+      <c r="D15" s="198"/>
+      <c r="E15" s="199"/>
+      <c r="F15" s="197" t="s">
         <v>8</v>
       </c>
-      <c r="G15" s="204"/>
-      <c r="H15" s="204"/>
-      <c r="I15" s="204"/>
+      <c r="G15" s="198"/>
+      <c r="H15" s="198"/>
+      <c r="I15" s="198"/>
       <c r="J15" s="19"/>
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
@@ -2235,7 +2235,7 @@
       <c r="Z15" s="7"/>
       <c r="AA15" s="7"/>
     </row>
-    <row r="16" spans="2:30" ht="1.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:30" ht="1.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="161" t="s">
         <v>17</v>
       </c>
@@ -2264,19 +2264,19 @@
       <c r="Z16" s="7"/>
       <c r="AA16" s="7"/>
     </row>
-    <row r="17" spans="2:30" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="212" t="s">
+    <row r="17" spans="2:30" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="209" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="213"/>
-      <c r="D17" s="213"/>
-      <c r="E17" s="214"/>
-      <c r="F17" s="212" t="s">
+      <c r="C17" s="210"/>
+      <c r="D17" s="210"/>
+      <c r="E17" s="211"/>
+      <c r="F17" s="209" t="s">
         <v>34</v>
       </c>
-      <c r="G17" s="213"/>
-      <c r="H17" s="213"/>
-      <c r="I17" s="213"/>
+      <c r="G17" s="210"/>
+      <c r="H17" s="210"/>
+      <c r="I17" s="210"/>
       <c r="J17" s="19"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
@@ -2293,24 +2293,24 @@
       <c r="Z17" s="7"/>
       <c r="AA17" s="7"/>
     </row>
-    <row r="18" spans="2:30" ht="37.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="215" t="s">
+    <row r="18" spans="2:30" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="212" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="216"/>
+      <c r="C18" s="213"/>
       <c r="D18" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="216" t="s">
+      <c r="E18" s="213" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="216"/>
-      <c r="G18" s="216"/>
+      <c r="F18" s="213"/>
+      <c r="G18" s="213"/>
       <c r="H18" s="20" t="s">
-        <v>35</v>
+        <v>115</v>
       </c>
       <c r="I18" s="20" t="s">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="J18" s="21"/>
       <c r="N18" s="7"/>
@@ -2328,19 +2328,19 @@
       <c r="Z18" s="7"/>
       <c r="AA18" s="7"/>
     </row>
-    <row r="19" spans="2:30" ht="25.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="217" t="s">
+    <row r="19" spans="2:30" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="214" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="218"/>
+      <c r="C19" s="215"/>
       <c r="D19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="219" t="s">
+      <c r="E19" s="216" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="220"/>
-      <c r="G19" s="220"/>
+      <c r="F19" s="217"/>
+      <c r="G19" s="217"/>
       <c r="H19" s="187" t="s">
         <v>12</v>
       </c>
@@ -2366,7 +2366,7 @@
       <c r="AC19" s="7"/>
       <c r="AD19" s="7"/>
     </row>
-    <row r="20" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="183"/>
       <c r="C20" s="184"/>
       <c r="D20" s="184"/>
@@ -2394,7 +2394,7 @@
       <c r="AC20" s="7"/>
       <c r="AD20" s="7"/>
     </row>
-    <row r="21" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="183"/>
       <c r="C21" s="184"/>
       <c r="D21" s="184"/>
@@ -2422,7 +2422,7 @@
       <c r="AC21" s="7"/>
       <c r="AD21" s="7"/>
     </row>
-    <row r="22" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="183"/>
       <c r="C22" s="184"/>
       <c r="D22" s="184"/>
@@ -2450,7 +2450,7 @@
       <c r="AC22" s="7"/>
       <c r="AD22" s="7"/>
     </row>
-    <row r="23" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="183"/>
       <c r="C23" s="184"/>
       <c r="D23" s="184"/>
@@ -2478,7 +2478,7 @@
       <c r="AC23" s="7"/>
       <c r="AD23" s="7"/>
     </row>
-    <row r="24" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="183"/>
       <c r="C24" s="184"/>
       <c r="D24" s="184"/>
@@ -2506,7 +2506,7 @@
       <c r="AC24" s="7"/>
       <c r="AD24" s="7"/>
     </row>
-    <row r="25" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="183"/>
       <c r="C25" s="184"/>
       <c r="D25" s="184"/>
@@ -2534,7 +2534,7 @@
       <c r="AC25" s="7"/>
       <c r="AD25" s="7"/>
     </row>
-    <row r="26" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="183"/>
       <c r="C26" s="184"/>
       <c r="D26" s="184"/>
@@ -2562,7 +2562,7 @@
       <c r="AC26" s="7"/>
       <c r="AD26" s="7"/>
     </row>
-    <row r="27" spans="2:30" ht="0.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="183"/>
       <c r="C27" s="184"/>
       <c r="D27" s="184"/>
@@ -2590,7 +2590,7 @@
       <c r="AC27" s="7"/>
       <c r="AD27" s="7"/>
     </row>
-    <row r="28" spans="2:30" ht="25.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:30" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="150" t="s">
         <v>17</v>
       </c>
@@ -2622,7 +2622,7 @@
       <c r="AC28" s="7"/>
       <c r="AD28" s="7"/>
     </row>
-    <row r="29" spans="2:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="189" t="s">
         <v>17</v>
       </c>
@@ -2654,7 +2654,7 @@
       <c r="AC29" s="7"/>
       <c r="AD29" s="7"/>
     </row>
-    <row r="30" spans="2:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="171" t="s">
         <v>17</v>
       </c>
@@ -2686,7 +2686,7 @@
       <c r="AC30" s="7"/>
       <c r="AD30" s="7"/>
     </row>
-    <row r="31" spans="2:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="171" t="s">
         <v>17</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="AC31" s="7"/>
       <c r="AD31" s="7"/>
     </row>
-    <row r="32" spans="2:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
         <v>17</v>
       </c>
@@ -2750,7 +2750,7 @@
       <c r="AC32" s="7"/>
       <c r="AD32" s="7"/>
     </row>
-    <row r="33" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="171" t="s">
         <v>17</v>
       </c>
@@ -2782,7 +2782,7 @@
       <c r="AC33" s="7"/>
       <c r="AD33" s="7"/>
     </row>
-    <row r="34" spans="1:30" s="27" customFormat="1" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:30" s="27" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="16" t="s">
         <v>17</v>
       </c>
@@ -2797,7 +2797,7 @@
       <c r="I34" s="18"/>
       <c r="J34" s="154"/>
     </row>
-    <row r="35" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="169" t="s">
         <v>17</v>
       </c>
@@ -2829,19 +2829,19 @@
       <c r="AC35" s="7"/>
       <c r="AD35" s="7"/>
     </row>
-    <row r="36" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B36" s="203" t="s">
-        <v>17</v>
-      </c>
-      <c r="C36" s="204"/>
-      <c r="D36" s="204"/>
-      <c r="E36" s="204"/>
-      <c r="F36" s="203" t="s">
-        <v>17</v>
-      </c>
-      <c r="G36" s="204"/>
-      <c r="H36" s="204"/>
-      <c r="I36" s="205"/>
+    <row r="36" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="197" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="198"/>
+      <c r="D36" s="198"/>
+      <c r="E36" s="198"/>
+      <c r="F36" s="197" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" s="198"/>
+      <c r="H36" s="198"/>
+      <c r="I36" s="199"/>
       <c r="J36" s="13"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
@@ -2861,7 +2861,7 @@
       <c r="AC36" s="7"/>
       <c r="AD36" s="7"/>
     </row>
-    <row r="37" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="16" t="s">
         <v>17</v>
       </c>
@@ -2893,7 +2893,7 @@
       <c r="AC37" s="7"/>
       <c r="AD37" s="7"/>
     </row>
-    <row r="38" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="16" t="s">
         <v>17</v>
       </c>
@@ -2925,37 +2925,37 @@
       <c r="AC38" s="7"/>
       <c r="AD38" s="7"/>
     </row>
-    <row r="39" spans="1:30" s="27" customFormat="1" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B39" s="221" t="s">
-        <v>84</v>
-      </c>
-      <c r="C39" s="222"/>
-      <c r="D39" s="222"/>
-      <c r="E39" s="222"/>
-      <c r="F39" s="221" t="s">
-        <v>84</v>
-      </c>
-      <c r="G39" s="222"/>
-      <c r="H39" s="222"/>
-      <c r="I39" s="223"/>
+    <row r="39" spans="1:30" s="27" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="204" t="s">
+        <v>80</v>
+      </c>
+      <c r="C39" s="205"/>
+      <c r="D39" s="205"/>
+      <c r="E39" s="205"/>
+      <c r="F39" s="204" t="s">
+        <v>80</v>
+      </c>
+      <c r="G39" s="205"/>
+      <c r="H39" s="205"/>
+      <c r="I39" s="206"/>
       <c r="J39" s="154"/>
     </row>
-    <row r="40" spans="1:30" s="27" customFormat="1" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B40" s="209" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="210"/>
-      <c r="D40" s="210"/>
-      <c r="E40" s="210"/>
-      <c r="F40" s="203" t="s">
-        <v>17</v>
-      </c>
-      <c r="G40" s="204"/>
-      <c r="H40" s="204"/>
-      <c r="I40" s="205"/>
+    <row r="40" spans="1:30" s="27" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="207" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="208"/>
+      <c r="D40" s="208"/>
+      <c r="E40" s="208"/>
+      <c r="F40" s="197" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="198"/>
+      <c r="H40" s="198"/>
+      <c r="I40" s="199"/>
       <c r="J40" s="154"/>
     </row>
-    <row r="41" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="169" t="s">
         <v>17</v>
       </c>
@@ -2987,22 +2987,22 @@
       <c r="AC41" s="7"/>
       <c r="AD41" s="7"/>
     </row>
-    <row r="42" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B42" s="203" t="s">
-        <v>17</v>
-      </c>
-      <c r="C42" s="204"/>
-      <c r="D42" s="204"/>
-      <c r="E42" s="204"/>
-      <c r="F42" s="203" t="s">
-        <v>17</v>
-      </c>
-      <c r="G42" s="204"/>
-      <c r="H42" s="204"/>
-      <c r="I42" s="205"/>
+    <row r="42" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="197" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="198"/>
+      <c r="D42" s="198"/>
+      <c r="E42" s="198"/>
+      <c r="F42" s="197" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" s="198"/>
+      <c r="H42" s="198"/>
+      <c r="I42" s="199"/>
       <c r="J42" s="6"/>
     </row>
-    <row r="43" spans="1:30" ht="24.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="194" t="s">
         <v>14</v>
       </c>
@@ -3017,7 +3017,7 @@
       <c r="I43" s="157"/>
       <c r="J43" s="6"/>
     </row>
-    <row r="44" spans="1:30" ht="4.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:30" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="170"/>
       <c r="B44" s="169"/>
       <c r="C44" s="5"/>
@@ -3029,7 +3029,7 @@
       <c r="I44" s="42"/>
       <c r="J44" s="6"/>
     </row>
-    <row r="45" spans="1:30" ht="19.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:30" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="158" t="s">
         <v>22</v>
       </c>
@@ -3044,19 +3044,19 @@
       <c r="I45" s="42"/>
       <c r="J45" s="6"/>
     </row>
-    <row r="46" spans="1:30" s="27" customFormat="1" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B46" s="224" t="s">
+    <row r="46" spans="1:30" s="27" customFormat="1" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="200" t="s">
+        <v>93</v>
+      </c>
+      <c r="C46" s="201"/>
+      <c r="D46" s="201"/>
+      <c r="E46" s="201"/>
+      <c r="F46" s="200" t="s">
         <v>97</v>
       </c>
-      <c r="C46" s="225"/>
-      <c r="D46" s="225"/>
-      <c r="E46" s="225"/>
-      <c r="F46" s="224" t="s">
-        <v>101</v>
-      </c>
-      <c r="G46" s="225"/>
-      <c r="H46" s="225"/>
-      <c r="I46" s="226"/>
+      <c r="G46" s="201"/>
+      <c r="H46" s="201"/>
+      <c r="I46" s="202"/>
       <c r="J46" s="26"/>
       <c r="N46" s="28"/>
       <c r="O46" s="28"/>
@@ -3076,97 +3076,97 @@
       <c r="AC46" s="28"/>
       <c r="AD46" s="28"/>
     </row>
-    <row r="47" spans="1:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B47" s="203" t="s">
+    <row r="47" spans="1:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="197" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" s="198"/>
+      <c r="D47" s="198"/>
+      <c r="E47" s="198"/>
+      <c r="F47" s="197" t="s">
         <v>98</v>
       </c>
-      <c r="C47" s="204"/>
-      <c r="D47" s="204"/>
-      <c r="E47" s="204"/>
-      <c r="F47" s="203" t="s">
+      <c r="G47" s="198"/>
+      <c r="H47" s="198"/>
+      <c r="I47" s="199"/>
+      <c r="J47" s="16"/>
+    </row>
+    <row r="48" spans="1:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="197" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" s="198"/>
+      <c r="D48" s="198"/>
+      <c r="E48" s="199"/>
+      <c r="F48" s="197" t="s">
+        <v>99</v>
+      </c>
+      <c r="G48" s="198"/>
+      <c r="H48" s="198"/>
+      <c r="I48" s="198"/>
+      <c r="J48" s="16"/>
+    </row>
+    <row r="49" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="197" t="s">
+        <v>101</v>
+      </c>
+      <c r="C49" s="198"/>
+      <c r="D49" s="198"/>
+      <c r="E49" s="199"/>
+      <c r="F49" s="197" t="s">
         <v>102</v>
       </c>
-      <c r="G47" s="204"/>
-      <c r="H47" s="204"/>
-      <c r="I47" s="205"/>
-      <c r="J47" s="16"/>
-    </row>
-    <row r="48" spans="1:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B48" s="203" t="s">
+      <c r="G49" s="198"/>
+      <c r="H49" s="198"/>
+      <c r="I49" s="198"/>
+      <c r="J49" s="16"/>
+    </row>
+    <row r="50" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="197" t="s">
+        <v>103</v>
+      </c>
+      <c r="C50" s="198"/>
+      <c r="D50" s="198"/>
+      <c r="E50" s="199"/>
+      <c r="F50" s="197" t="s">
+        <v>103</v>
+      </c>
+      <c r="G50" s="198"/>
+      <c r="H50" s="198"/>
+      <c r="I50" s="198"/>
+      <c r="J50" s="16"/>
+    </row>
+    <row r="51" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="197" t="s">
         <v>104</v>
       </c>
-      <c r="C48" s="204"/>
-      <c r="D48" s="204"/>
-      <c r="E48" s="205"/>
-      <c r="F48" s="203" t="s">
-        <v>103</v>
-      </c>
-      <c r="G48" s="204"/>
-      <c r="H48" s="204"/>
-      <c r="I48" s="204"/>
-      <c r="J48" s="16"/>
-    </row>
-    <row r="49" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B49" s="203" t="s">
+      <c r="C51" s="198"/>
+      <c r="D51" s="198"/>
+      <c r="E51" s="199"/>
+      <c r="F51" s="197" t="s">
         <v>105</v>
       </c>
-      <c r="C49" s="204"/>
-      <c r="D49" s="204"/>
-      <c r="E49" s="205"/>
-      <c r="F49" s="203" t="s">
+      <c r="G51" s="198"/>
+      <c r="H51" s="198"/>
+      <c r="I51" s="198"/>
+      <c r="J51" s="16"/>
+    </row>
+    <row r="52" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="197" t="s">
         <v>106</v>
       </c>
-      <c r="G49" s="204"/>
-      <c r="H49" s="204"/>
-      <c r="I49" s="204"/>
-      <c r="J49" s="16"/>
-    </row>
-    <row r="50" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B50" s="203" t="s">
+      <c r="C52" s="198"/>
+      <c r="D52" s="198"/>
+      <c r="E52" s="199"/>
+      <c r="F52" s="197" t="s">
         <v>107</v>
       </c>
-      <c r="C50" s="204"/>
-      <c r="D50" s="204"/>
-      <c r="E50" s="205"/>
-      <c r="F50" s="203" t="s">
-        <v>107</v>
-      </c>
-      <c r="G50" s="204"/>
-      <c r="H50" s="204"/>
-      <c r="I50" s="204"/>
-      <c r="J50" s="16"/>
-    </row>
-    <row r="51" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B51" s="203" t="s">
-        <v>108</v>
-      </c>
-      <c r="C51" s="204"/>
-      <c r="D51" s="204"/>
-      <c r="E51" s="205"/>
-      <c r="F51" s="203" t="s">
-        <v>109</v>
-      </c>
-      <c r="G51" s="204"/>
-      <c r="H51" s="204"/>
-      <c r="I51" s="204"/>
-      <c r="J51" s="16"/>
-    </row>
-    <row r="52" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B52" s="203" t="s">
-        <v>110</v>
-      </c>
-      <c r="C52" s="204"/>
-      <c r="D52" s="204"/>
-      <c r="E52" s="205"/>
-      <c r="F52" s="203" t="s">
-        <v>111</v>
-      </c>
-      <c r="G52" s="204"/>
-      <c r="H52" s="204"/>
-      <c r="I52" s="204"/>
+      <c r="G52" s="198"/>
+      <c r="H52" s="198"/>
+      <c r="I52" s="198"/>
       <c r="J52" s="16"/>
     </row>
-    <row r="53" spans="2:30" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:30" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="169" t="s">
         <v>28</v>
       </c>
@@ -3181,19 +3181,19 @@
       <c r="I53" s="17"/>
       <c r="J53" s="16"/>
     </row>
-    <row r="54" spans="2:30" s="27" customFormat="1" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B54" s="224" t="s">
-        <v>97</v>
-      </c>
-      <c r="C54" s="225"/>
-      <c r="D54" s="225"/>
-      <c r="E54" s="226"/>
-      <c r="F54" s="224" t="s">
-        <v>97</v>
-      </c>
-      <c r="G54" s="227"/>
-      <c r="H54" s="227"/>
-      <c r="I54" s="227"/>
+    <row r="54" spans="2:30" s="27" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="200" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="201"/>
+      <c r="D54" s="201"/>
+      <c r="E54" s="202"/>
+      <c r="F54" s="200" t="s">
+        <v>93</v>
+      </c>
+      <c r="G54" s="203"/>
+      <c r="H54" s="203"/>
+      <c r="I54" s="203"/>
       <c r="J54" s="26"/>
       <c r="N54" s="28"/>
       <c r="O54" s="28"/>
@@ -3213,22 +3213,22 @@
       <c r="AC54" s="28"/>
       <c r="AD54" s="28"/>
     </row>
-    <row r="55" spans="2:30" ht="26.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B55" s="203" t="s">
-        <v>112</v>
-      </c>
-      <c r="C55" s="204"/>
-      <c r="D55" s="204"/>
-      <c r="E55" s="205"/>
-      <c r="F55" s="203" t="s">
-        <v>112</v>
-      </c>
-      <c r="G55" s="204"/>
-      <c r="H55" s="204"/>
-      <c r="I55" s="204"/>
+    <row r="55" spans="2:30" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="197" t="s">
+        <v>108</v>
+      </c>
+      <c r="C55" s="198"/>
+      <c r="D55" s="198"/>
+      <c r="E55" s="199"/>
+      <c r="F55" s="197" t="s">
+        <v>108</v>
+      </c>
+      <c r="G55" s="198"/>
+      <c r="H55" s="198"/>
+      <c r="I55" s="198"/>
       <c r="J55" s="16"/>
     </row>
-    <row r="56" spans="2:30" ht="1.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:30" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="16"/>
       <c r="C56" s="25"/>
       <c r="D56" s="25"/>
@@ -3241,22 +3241,22 @@
       <c r="I56" s="17"/>
       <c r="J56" s="16"/>
     </row>
-    <row r="57" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C57" s="23"/>
       <c r="D57" s="23"/>
       <c r="E57" s="29"/>
       <c r="F57" s="22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G57" s="23"/>
       <c r="H57" s="30"/>
       <c r="I57" s="30"/>
       <c r="J57" s="16"/>
     </row>
-    <row r="58" spans="2:30" ht="1.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:30" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="31"/>
       <c r="C58" s="25" t="s">
         <v>17</v>
@@ -3269,7 +3269,7 @@
       <c r="I58" s="30"/>
       <c r="J58" s="16"/>
     </row>
-    <row r="59" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="22" t="s">
         <v>18</v>
       </c>
@@ -3284,67 +3284,67 @@
       <c r="I59" s="30"/>
       <c r="J59" s="16"/>
     </row>
-    <row r="60" spans="2:30" ht="26.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B60" s="203" t="s">
-        <v>105</v>
-      </c>
-      <c r="C60" s="204"/>
-      <c r="D60" s="204"/>
-      <c r="E60" s="205"/>
-      <c r="F60" s="203" t="s">
-        <v>105</v>
-      </c>
-      <c r="G60" s="204"/>
-      <c r="H60" s="204"/>
-      <c r="I60" s="205"/>
+    <row r="60" spans="2:30" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="197" t="s">
+        <v>101</v>
+      </c>
+      <c r="C60" s="198"/>
+      <c r="D60" s="198"/>
+      <c r="E60" s="199"/>
+      <c r="F60" s="197" t="s">
+        <v>101</v>
+      </c>
+      <c r="G60" s="198"/>
+      <c r="H60" s="198"/>
+      <c r="I60" s="199"/>
       <c r="J60" s="16"/>
     </row>
-    <row r="61" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="22" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C61" s="23"/>
       <c r="D61" s="23"/>
       <c r="E61" s="24"/>
       <c r="F61" s="23" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G61" s="30"/>
       <c r="H61" s="30"/>
       <c r="I61" s="30"/>
       <c r="J61" s="16"/>
     </row>
-    <row r="62" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="22" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C62" s="23"/>
       <c r="D62" s="23"/>
       <c r="E62" s="24"/>
       <c r="F62" s="23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G62" s="30"/>
       <c r="H62" s="30"/>
       <c r="I62" s="30"/>
       <c r="J62" s="16"/>
     </row>
-    <row r="63" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="22" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C63" s="23"/>
       <c r="D63" s="23"/>
       <c r="E63" s="24"/>
       <c r="F63" s="23" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G63" s="23"/>
       <c r="H63" s="23"/>
       <c r="I63" s="23"/>
       <c r="J63" s="16"/>
     </row>
-    <row r="64" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="16"/>
       <c r="C64" s="28" t="s">
         <v>17</v>
@@ -3359,7 +3359,7 @@
       <c r="I64" s="25"/>
       <c r="J64" s="16"/>
     </row>
-    <row r="65" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="32" t="s">
         <v>19</v>
       </c>
@@ -3374,7 +3374,7 @@
       <c r="I65" s="34"/>
       <c r="J65" s="12"/>
     </row>
-    <row r="66" spans="2:10" ht="10.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:10" ht="10.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="35"/>
       <c r="C66" s="36" t="s">
         <v>17</v>
@@ -3391,7 +3391,7 @@
       <c r="I66" s="38"/>
       <c r="J66" s="12"/>
     </row>
-    <row r="67" spans="2:10" ht="7.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:10" ht="7.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="12"/>
       <c r="C67" s="40"/>
       <c r="D67" s="40"/>
@@ -3402,7 +3402,7 @@
       <c r="I67" s="12"/>
       <c r="J67" s="12"/>
     </row>
-    <row r="68" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="12"/>
       <c r="C68" s="40"/>
       <c r="D68" s="40"/>
@@ -3413,7 +3413,7 @@
       <c r="I68" s="12"/>
       <c r="J68" s="12"/>
     </row>
-    <row r="69" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="12"/>
       <c r="C69" s="40"/>
       <c r="D69" s="40"/>
@@ -3424,7 +3424,7 @@
       <c r="I69" s="12"/>
       <c r="J69" s="12"/>
     </row>
-    <row r="70" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="12"/>
       <c r="C70" s="40"/>
       <c r="D70" s="40"/>
@@ -3435,7 +3435,7 @@
       <c r="I70" s="12"/>
       <c r="J70" s="12"/>
     </row>
-    <row r="71" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="12"/>
       <c r="C71" s="40"/>
       <c r="D71" s="40"/>
@@ -3446,7 +3446,7 @@
       <c r="I71" s="12"/>
       <c r="J71" s="12"/>
     </row>
-    <row r="72" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="12"/>
       <c r="C72" s="40"/>
       <c r="D72" s="40"/>
@@ -3457,7 +3457,7 @@
       <c r="I72" s="12"/>
       <c r="J72" s="12"/>
     </row>
-    <row r="73" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="12"/>
       <c r="C73" s="40"/>
       <c r="D73" s="40"/>
@@ -3468,7 +3468,7 @@
       <c r="I73" s="12"/>
       <c r="J73" s="12"/>
     </row>
-    <row r="74" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="12"/>
       <c r="C74" s="40"/>
       <c r="D74" s="40"/>
@@ -3479,7 +3479,7 @@
       <c r="I74" s="12"/>
       <c r="J74" s="12"/>
     </row>
-    <row r="75" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="12"/>
       <c r="C75" s="40"/>
       <c r="D75" s="40"/>
@@ -3490,7 +3490,7 @@
       <c r="I75" s="12"/>
       <c r="J75" s="12"/>
     </row>
-    <row r="76" spans="2:10" ht="7.25" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:10" ht="7.35" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="12"/>
       <c r="C76" s="40"/>
       <c r="D76" s="40"/>
@@ -3501,20 +3501,56 @@
       <c r="I76" s="12"/>
       <c r="J76" s="12"/>
     </row>
-    <row r="77" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="78" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="79" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="80" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="81" spans="6:7" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="82" spans="6:7" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="90" spans="6:7" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="2:10" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="6:7" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="6:7" ht="3.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F90" s="7"/>
       <c r="G90" s="7"/>
     </row>
-    <row r="95" spans="6:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="102" ht="43.5" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="95" spans="6:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="43.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="B9:E10"/>
+    <mergeCell ref="F9:I10"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="F47:I47"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="F48:I48"/>
     <mergeCell ref="B60:E60"/>
@@ -3531,42 +3567,6 @@
     <mergeCell ref="F51:I51"/>
     <mergeCell ref="B52:E52"/>
     <mergeCell ref="F52:I52"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="F36:I36"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B9:E10"/>
-    <mergeCell ref="F9:I10"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="D19:E31 J19:J31 E32:E33 B33">
     <cfRule type="notContainsBlanks" dxfId="3" priority="2">
@@ -3593,7 +3593,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.35433070866141736" bottom="0.15748031496062992" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="74" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="76" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3604,36 +3604,36 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AC55"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1" customWidth="1"/>
-    <col min="2" max="2" width="11.73046875" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14.3984375" customWidth="1"/>
-    <col min="5" max="5" width="8.46484375" customWidth="1"/>
-    <col min="6" max="6" width="19.86328125" customWidth="1"/>
-    <col min="7" max="7" width="0.9296875" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" customWidth="1"/>
-    <col min="10" max="10" width="14.19921875" customWidth="1"/>
-    <col min="11" max="11" width="5.59765625" customWidth="1"/>
-    <col min="12" max="12" width="7.1328125" customWidth="1"/>
-    <col min="13" max="13" width="15.53125" customWidth="1"/>
-    <col min="14" max="14" width="0.59765625" customWidth="1"/>
-    <col min="15" max="18" width="9.1328125" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" customWidth="1"/>
+    <col min="7" max="7" width="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" customWidth="1"/>
+    <col min="11" max="11" width="5.5703125" customWidth="1"/>
+    <col min="12" max="12" width="7.140625" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" customWidth="1"/>
+    <col min="14" max="14" width="0.5703125" customWidth="1"/>
+    <col min="15" max="18" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="3" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" ht="3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="45"/>
       <c r="G1" s="142" t="s">
         <v>17</v>
       </c>
       <c r="N1" s="47"/>
     </row>
-    <row r="2" spans="1:14" ht="37.9" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:14" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="76"/>
       <c r="B2" s="104" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C2" s="104"/>
       <c r="D2" s="104"/>
@@ -3641,7 +3641,7 @@
       <c r="F2" s="104"/>
       <c r="G2" s="104"/>
       <c r="H2" s="107" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I2" s="104"/>
       <c r="J2" s="104"/>
@@ -3650,10 +3650,10 @@
       <c r="M2" s="104"/>
       <c r="N2" s="47"/>
     </row>
-    <row r="3" spans="1:14" ht="33.4" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:14" ht="33.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
       <c r="B3" s="105" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C3" s="105"/>
       <c r="D3" s="105"/>
@@ -3661,7 +3661,7 @@
       <c r="F3" s="106"/>
       <c r="G3" s="106"/>
       <c r="H3" s="108" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="I3" s="105"/>
       <c r="J3" s="105"/>
@@ -3670,10 +3670,10 @@
       <c r="M3" s="105"/>
       <c r="N3" s="47"/>
     </row>
-    <row r="4" spans="1:14" s="73" customFormat="1" ht="23.35" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" s="73" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75"/>
       <c r="B4" s="105" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C4" s="105"/>
       <c r="D4" s="105"/>
@@ -3681,7 +3681,7 @@
       <c r="F4" s="105"/>
       <c r="G4" s="105"/>
       <c r="H4" s="108" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="I4" s="105"/>
       <c r="J4" s="105"/>
@@ -3690,10 +3690,10 @@
       <c r="M4" s="105"/>
       <c r="N4" s="71"/>
     </row>
-    <row r="5" spans="1:14" s="73" customFormat="1" ht="27.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" s="73" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="74"/>
       <c r="B5" s="105" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C5" s="105"/>
       <c r="D5" s="105"/>
@@ -3701,7 +3701,7 @@
       <c r="F5" s="105"/>
       <c r="G5" s="105"/>
       <c r="H5" s="108" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I5" s="105"/>
       <c r="J5" s="105"/>
@@ -3710,10 +3710,10 @@
       <c r="M5" s="105"/>
       <c r="N5" s="71"/>
     </row>
-    <row r="6" spans="1:14" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="45"/>
       <c r="B6" s="95" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C6" s="95"/>
       <c r="D6" s="95"/>
@@ -3730,7 +3730,7 @@
       <c r="M6" s="84"/>
       <c r="N6" s="47"/>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="45"/>
       <c r="B7" s="98" t="s">
         <v>23</v>
@@ -3750,7 +3750,7 @@
       <c r="M7" s="84"/>
       <c r="N7" s="47"/>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="45"/>
       <c r="B8" s="110" t="s">
         <v>3</v>
@@ -3770,7 +3770,7 @@
       <c r="M8" s="84"/>
       <c r="N8" s="47"/>
     </row>
-    <row r="9" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="45"/>
       <c r="B9" s="111" t="s">
         <v>28</v>
@@ -3781,7 +3781,7 @@
       <c r="F9" s="111"/>
       <c r="G9" s="111"/>
       <c r="H9" s="89" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I9" s="84"/>
       <c r="J9" s="84"/>
@@ -3790,7 +3790,7 @@
       <c r="M9" s="84"/>
       <c r="N9" s="47"/>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="45"/>
       <c r="B10" s="98" t="s">
         <v>5</v>
@@ -3810,7 +3810,7 @@
       <c r="M10" s="84"/>
       <c r="N10" s="47"/>
     </row>
-    <row r="11" spans="1:14" ht="31.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" ht="31.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="45"/>
       <c r="B11" s="88" t="s">
         <v>6</v>
@@ -3830,10 +3830,10 @@
       <c r="M11" s="88"/>
       <c r="N11" s="47"/>
     </row>
-    <row r="12" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="45"/>
       <c r="B12" s="111" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C12" s="111"/>
       <c r="D12" s="111"/>
@@ -3841,7 +3841,7 @@
       <c r="F12" s="111"/>
       <c r="G12" s="111"/>
       <c r="H12" s="82" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="I12" s="83"/>
       <c r="J12" s="83"/>
@@ -3850,7 +3850,7 @@
       <c r="M12" s="84"/>
       <c r="N12" s="47"/>
     </row>
-    <row r="13" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="45"/>
       <c r="B13" s="98" t="s">
         <v>5</v>
@@ -3870,7 +3870,7 @@
       <c r="M13" s="84"/>
       <c r="N13" s="47"/>
     </row>
-    <row r="14" spans="1:14" ht="54" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="45"/>
       <c r="B14" s="151" t="s">
         <v>6</v>
@@ -3890,35 +3890,35 @@
       <c r="M14" s="88"/>
       <c r="N14" s="47"/>
     </row>
-    <row r="15" spans="1:14" ht="32.65" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" ht="32.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="72"/>
       <c r="B15" s="230" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C15" s="231"/>
       <c r="D15" s="90" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E15" s="90"/>
       <c r="F15" s="90" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G15" s="90"/>
       <c r="H15" s="91" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I15" s="90"/>
       <c r="J15" s="112" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="K15" s="112"/>
       <c r="L15" s="136" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="M15" s="136"/>
       <c r="N15" s="47"/>
     </row>
-    <row r="16" spans="1:14" ht="29.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="45"/>
       <c r="B16" s="92" t="s">
         <v>17</v>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="E16" s="93"/>
       <c r="F16" s="129" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G16" s="93"/>
       <c r="H16" s="153" t="s">
@@ -3941,40 +3941,40 @@
       </c>
       <c r="K16" s="94"/>
       <c r="L16" s="137" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="M16" s="137"/>
       <c r="N16" s="47"/>
     </row>
-    <row r="17" spans="1:29" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:29" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45"/>
       <c r="B17" s="133" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C17" s="111"/>
       <c r="D17" s="130" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E17" s="115"/>
       <c r="F17" s="128" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G17" s="128"/>
       <c r="H17" s="89" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I17" s="84"/>
       <c r="J17" s="96" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="K17" s="84"/>
       <c r="L17" s="138" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="M17" s="139"/>
       <c r="N17" s="47"/>
     </row>
-    <row r="18" spans="1:29" ht="29.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:29" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="45"/>
       <c r="B18" s="110" t="s">
         <v>17</v>
@@ -4002,31 +4002,31 @@
       <c r="M18" s="137"/>
       <c r="N18" s="47"/>
     </row>
-    <row r="19" spans="1:29" ht="27.85" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:29" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="45"/>
       <c r="B19" s="133" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C19" s="116"/>
       <c r="D19" s="116" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E19" s="116"/>
       <c r="F19" s="116"/>
       <c r="G19" s="130"/>
       <c r="H19" s="133" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I19" s="113"/>
       <c r="J19" s="111" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="K19" s="111"/>
       <c r="L19" s="111"/>
       <c r="M19" s="111"/>
       <c r="N19" s="47"/>
     </row>
-    <row r="20" spans="1:29" ht="29.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:29" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="45"/>
       <c r="B20" s="93" t="s">
         <v>17</v>
@@ -4050,7 +4050,7 @@
       <c r="M20" s="94"/>
       <c r="N20" s="47"/>
     </row>
-    <row r="21" spans="1:29" s="69" customFormat="1" ht="22.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:29" s="69" customFormat="1" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="81"/>
       <c r="B21" s="100"/>
       <c r="C21" s="100"/>
@@ -4077,67 +4077,67 @@
       <c r="AB21"/>
       <c r="AC21"/>
     </row>
-    <row r="22" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="45"/>
       <c r="B22" s="49" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C22" s="117" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D22" s="117"/>
       <c r="E22" s="117"/>
       <c r="F22" s="135"/>
       <c r="G22" s="117"/>
       <c r="H22" s="49" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I22" s="68" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J22" s="67" t="s">
-        <v>50</v>
+        <v>113</v>
       </c>
       <c r="K22" s="117" t="s">
-        <v>49</v>
+        <v>114</v>
       </c>
       <c r="L22" s="117"/>
       <c r="M22" s="49" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="N22" s="47"/>
     </row>
-    <row r="23" spans="1:29" ht="52.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:29" ht="52.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="45"/>
       <c r="B23" s="124" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C23" s="228" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D23" s="228"/>
       <c r="E23" s="228"/>
       <c r="F23" s="228"/>
       <c r="G23" s="125"/>
       <c r="H23" s="126" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I23" s="66" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J23" s="65">
         <v>14</v>
       </c>
       <c r="K23" s="229" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="L23" s="229"/>
       <c r="M23" s="64" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="N23" s="47"/>
     </row>
-    <row r="24" spans="1:29" ht="49.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:29" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="45"/>
       <c r="C24" s="122"/>
       <c r="D24" s="122"/>
@@ -4145,10 +4145,10 @@
       <c r="F24" s="122"/>
       <c r="G24" s="122"/>
       <c r="H24" s="123" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I24" s="63" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J24" s="62">
         <v>14</v>
@@ -4158,11 +4158,11 @@
       </c>
       <c r="L24" s="127"/>
       <c r="M24" s="77" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="N24" s="47"/>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="45"/>
       <c r="B25" s="56"/>
       <c r="C25" s="56"/>
@@ -4178,7 +4178,7 @@
       <c r="M25" s="61"/>
       <c r="N25" s="47"/>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="45"/>
       <c r="B26" s="56"/>
       <c r="C26" s="56"/>
@@ -4194,7 +4194,7 @@
       <c r="M26" s="61"/>
       <c r="N26" s="47"/>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="45"/>
       <c r="B27" s="56"/>
       <c r="C27" s="56"/>
@@ -4210,7 +4210,7 @@
       <c r="M27" s="61"/>
       <c r="N27" s="47"/>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A28" s="45"/>
       <c r="B28" s="56"/>
       <c r="C28" s="56"/>
@@ -4226,7 +4226,7 @@
       <c r="M28" s="61"/>
       <c r="N28" s="47"/>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A29" s="45"/>
       <c r="B29" s="56"/>
       <c r="C29" s="56"/>
@@ -4241,7 +4241,7 @@
       <c r="M29" s="61"/>
       <c r="N29" s="47"/>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A30" s="45"/>
       <c r="B30" s="56"/>
       <c r="C30" s="56"/>
@@ -4257,7 +4257,7 @@
       <c r="M30" s="61"/>
       <c r="N30" s="47"/>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A31" s="45"/>
       <c r="D31" s="56"/>
       <c r="E31" s="56"/>
@@ -4271,7 +4271,7 @@
       <c r="M31" s="61"/>
       <c r="N31" s="47"/>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A32" s="45"/>
       <c r="B32" s="56"/>
       <c r="C32" s="56"/>
@@ -4287,7 +4287,7 @@
       <c r="M32" s="61"/>
       <c r="N32" s="47"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="45"/>
       <c r="B33" s="56"/>
       <c r="C33" s="56"/>
@@ -4303,7 +4303,7 @@
       <c r="M33" s="61"/>
       <c r="N33" s="47"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="45"/>
       <c r="B34" s="56"/>
       <c r="C34" s="56"/>
@@ -4319,7 +4319,7 @@
       <c r="M34" s="61"/>
       <c r="N34" s="47"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="45"/>
       <c r="B35" s="56"/>
       <c r="C35" s="56"/>
@@ -4335,7 +4335,7 @@
       <c r="M35" s="61"/>
       <c r="N35" s="47"/>
     </row>
-    <row r="36" spans="1:14" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:14" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="45"/>
       <c r="C36" s="56"/>
       <c r="D36" s="56"/>
@@ -4350,7 +4350,7 @@
       <c r="M36" s="50"/>
       <c r="N36" s="47"/>
     </row>
-    <row r="37" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="45"/>
       <c r="B37" s="79" t="s">
         <v>21</v>
@@ -4362,7 +4362,7 @@
       <c r="G37" s="59"/>
       <c r="H37" s="58"/>
       <c r="I37" s="119" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J37" s="118"/>
       <c r="K37" s="118"/>
@@ -4370,10 +4370,10 @@
       <c r="M37" s="118"/>
       <c r="N37" s="47"/>
     </row>
-    <row r="38" spans="1:14" ht="15.4" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:14" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="45"/>
       <c r="B38" s="80" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C38" s="56"/>
       <c r="D38" s="56"/>
@@ -4390,7 +4390,7 @@
       <c r="M38" s="50"/>
       <c r="N38" s="47"/>
     </row>
-    <row r="39" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="45"/>
       <c r="B39" s="80" t="s">
         <v>16</v>
@@ -4407,10 +4407,10 @@
       <c r="M39" s="50"/>
       <c r="N39" s="47"/>
     </row>
-    <row r="40" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="45"/>
       <c r="B40" s="80" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C40" s="56"/>
       <c r="D40" s="56"/>
@@ -4425,10 +4425,10 @@
       <c r="M40" s="50"/>
       <c r="N40" s="47"/>
     </row>
-    <row r="41" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="45"/>
       <c r="B41" s="146" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C41" s="56"/>
       <c r="D41" s="56"/>
@@ -4445,7 +4445,7 @@
       <c r="M41" s="50"/>
       <c r="N41" s="47"/>
     </row>
-    <row r="42" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="149"/>
       <c r="C42" s="56"/>
       <c r="D42" s="56"/>
@@ -4459,7 +4459,7 @@
       <c r="M42" s="50"/>
       <c r="N42" s="47"/>
     </row>
-    <row r="43" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="149"/>
       <c r="C43" s="56"/>
       <c r="D43" s="56"/>
@@ -4474,7 +4474,7 @@
       <c r="M43" s="50"/>
       <c r="N43" s="47"/>
     </row>
-    <row r="44" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="149"/>
       <c r="C44" s="56"/>
       <c r="D44" s="56"/>
@@ -4489,7 +4489,7 @@
       <c r="M44" s="50"/>
       <c r="N44" s="47"/>
     </row>
-    <row r="45" spans="1:14" s="52" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:14" s="52" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="145"/>
       <c r="B45" s="147"/>
       <c r="C45" s="55"/>
@@ -4505,12 +4505,12 @@
       <c r="M45" s="121"/>
       <c r="N45" s="78"/>
     </row>
-    <row r="46" spans="1:14" ht="0.85" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="47" spans="1:14" ht="0.85" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="48" spans="1:14" ht="0.85" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="49" ht="0.85" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="50" ht="0.85" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="55" ht="2.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="46" spans="1:14" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:14" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:14" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="2.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="C23:F23"/>

</xml_diff>

<commit_message>
update EXW storage, now it looks like FCA non-com
</commit_message>
<xml_diff>
--- a/templates/Export_Agreement.xlsx
+++ b/templates/Export_Agreement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tsAddin\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5428E2-66C5-4818-8E14-35FF8B822CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC90952D-2449-4E48-803D-7E38E7AD7514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6FC3AD6-F63C-4057-BD0B-525C27FA51AB}"/>
+    <workbookView xWindow="4125" yWindow="2835" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{B6FC3AD6-F63C-4057-BD0B-525C27FA51AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Export_Contract" sheetId="1" r:id="rId1"/>
@@ -822,7 +822,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="232">
+  <cellXfs count="233">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1084,9 +1084,6 @@
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1344,6 +1341,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1437,17 +1449,8 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1868,31 +1871,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:30" ht="2.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="143"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
     </row>
     <row r="2" spans="2:30" s="14" customFormat="1" ht="21.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="222" t="s">
+      <c r="B2" s="226" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="223"/>
-      <c r="D2" s="223"/>
-      <c r="E2" s="224"/>
-      <c r="F2" s="222" t="s">
+      <c r="C2" s="227"/>
+      <c r="D2" s="227"/>
+      <c r="E2" s="228"/>
+      <c r="F2" s="226" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="223"/>
-      <c r="H2" s="223"/>
-      <c r="I2" s="223"/>
-      <c r="J2" s="144"/>
+      <c r="G2" s="227"/>
+      <c r="H2" s="227"/>
+      <c r="I2" s="227"/>
+      <c r="J2" s="143"/>
       <c r="L2" s="8"/>
       <c r="N2" s="15"/>
       <c r="AA2" s="15"/>
@@ -1901,18 +1904,18 @@
       <c r="AD2" s="15"/>
     </row>
     <row r="3" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="225" t="s">
+      <c r="B3" s="229" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="226"/>
-      <c r="D3" s="226"/>
-      <c r="E3" s="227"/>
-      <c r="F3" s="225" t="s">
+      <c r="C3" s="230"/>
+      <c r="D3" s="230"/>
+      <c r="E3" s="231"/>
+      <c r="F3" s="229" t="s">
         <v>85</v>
       </c>
-      <c r="G3" s="226"/>
-      <c r="H3" s="226"/>
-      <c r="I3" s="226"/>
+      <c r="G3" s="230"/>
+      <c r="H3" s="230"/>
+      <c r="I3" s="230"/>
       <c r="J3" s="6"/>
       <c r="L3" s="8"/>
       <c r="O3" s="7"/>
@@ -1929,18 +1932,18 @@
       <c r="Z3" s="7"/>
     </row>
     <row r="4" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="225" t="s">
+      <c r="B4" s="229" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="226"/>
-      <c r="D4" s="226"/>
-      <c r="E4" s="227"/>
-      <c r="F4" s="225" t="s">
+      <c r="C4" s="230"/>
+      <c r="D4" s="230"/>
+      <c r="E4" s="231"/>
+      <c r="F4" s="229" t="s">
         <v>86</v>
       </c>
-      <c r="G4" s="226"/>
-      <c r="H4" s="226"/>
-      <c r="I4" s="226"/>
+      <c r="G4" s="230"/>
+      <c r="H4" s="230"/>
+      <c r="I4" s="230"/>
       <c r="J4" s="6"/>
       <c r="N4" s="10"/>
       <c r="O4" s="11"/>
@@ -1961,18 +1964,18 @@
       <c r="AD4" s="10"/>
     </row>
     <row r="5" spans="2:30" s="14" customFormat="1" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="218" t="s">
+      <c r="B5" s="222" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="219"/>
-      <c r="D5" s="219"/>
-      <c r="E5" s="220"/>
-      <c r="F5" s="218" t="s">
+      <c r="C5" s="223"/>
+      <c r="D5" s="223"/>
+      <c r="E5" s="224"/>
+      <c r="F5" s="222" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="219"/>
-      <c r="H5" s="219"/>
-      <c r="I5" s="219"/>
+      <c r="G5" s="223"/>
+      <c r="H5" s="223"/>
+      <c r="I5" s="223"/>
       <c r="J5" s="13"/>
       <c r="N5" s="15"/>
       <c r="AA5" s="15"/>
@@ -1981,18 +1984,18 @@
       <c r="AD5" s="15"/>
     </row>
     <row r="6" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="161" t="s">
+      <c r="B6" s="160" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="162"/>
-      <c r="D6" s="162"/>
-      <c r="E6" s="163"/>
-      <c r="F6" s="161" t="s">
+      <c r="C6" s="161"/>
+      <c r="D6" s="161"/>
+      <c r="E6" s="162"/>
+      <c r="F6" s="160" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="162"/>
-      <c r="H6" s="162"/>
-      <c r="I6" s="162"/>
+      <c r="G6" s="161"/>
+      <c r="H6" s="161"/>
+      <c r="I6" s="161"/>
       <c r="J6" s="43"/>
       <c r="L6" s="44"/>
       <c r="O6" s="7"/>
@@ -2009,18 +2012,18 @@
       <c r="Z6" s="7"/>
     </row>
     <row r="7" spans="2:30" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="161" t="s">
+      <c r="B7" s="160" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="164"/>
-      <c r="D7" s="164"/>
-      <c r="E7" s="165"/>
-      <c r="F7" s="161" t="s">
+      <c r="C7" s="163"/>
+      <c r="D7" s="163"/>
+      <c r="E7" s="164"/>
+      <c r="F7" s="160" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="164"/>
-      <c r="H7" s="164"/>
-      <c r="I7" s="164"/>
+      <c r="G7" s="163"/>
+      <c r="H7" s="163"/>
+      <c r="I7" s="163"/>
       <c r="J7" s="43"/>
       <c r="L7" s="44"/>
       <c r="O7" s="7"/>
@@ -2037,44 +2040,44 @@
       <c r="Z7" s="7"/>
     </row>
     <row r="8" spans="2:30" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="207" t="s">
+      <c r="B8" s="211" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="208"/>
-      <c r="D8" s="208"/>
-      <c r="E8" s="221"/>
-      <c r="F8" s="207" t="s">
+      <c r="C8" s="212"/>
+      <c r="D8" s="212"/>
+      <c r="E8" s="225"/>
+      <c r="F8" s="211" t="s">
         <v>90</v>
       </c>
-      <c r="G8" s="208"/>
-      <c r="H8" s="208"/>
-      <c r="I8" s="208"/>
+      <c r="G8" s="212"/>
+      <c r="H8" s="212"/>
+      <c r="I8" s="212"/>
       <c r="J8" s="19"/>
     </row>
     <row r="9" spans="2:30" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="197" t="s">
+      <c r="B9" s="201" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="198"/>
-      <c r="D9" s="198"/>
-      <c r="E9" s="199"/>
-      <c r="F9" s="197" t="s">
+      <c r="C9" s="202"/>
+      <c r="D9" s="202"/>
+      <c r="E9" s="203"/>
+      <c r="F9" s="201" t="s">
         <v>92</v>
       </c>
-      <c r="G9" s="198"/>
-      <c r="H9" s="198"/>
-      <c r="I9" s="199"/>
+      <c r="G9" s="202"/>
+      <c r="H9" s="202"/>
+      <c r="I9" s="203"/>
       <c r="J9" s="19"/>
     </row>
     <row r="10" spans="2:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="197"/>
-      <c r="C10" s="198"/>
-      <c r="D10" s="198"/>
-      <c r="E10" s="199"/>
-      <c r="F10" s="197"/>
-      <c r="G10" s="198"/>
-      <c r="H10" s="198"/>
-      <c r="I10" s="199"/>
+      <c r="B10" s="201"/>
+      <c r="C10" s="202"/>
+      <c r="D10" s="202"/>
+      <c r="E10" s="203"/>
+      <c r="F10" s="201"/>
+      <c r="G10" s="202"/>
+      <c r="H10" s="202"/>
+      <c r="I10" s="203"/>
       <c r="J10" s="19"/>
       <c r="N10" s="15"/>
       <c r="O10" s="7"/>
@@ -2095,18 +2098,18 @@
       <c r="AD10" s="15"/>
     </row>
     <row r="11" spans="2:30" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="158" t="s">
+      <c r="B11" s="157" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="159"/>
-      <c r="D11" s="159"/>
-      <c r="E11" s="160"/>
-      <c r="F11" s="158" t="s">
+      <c r="C11" s="158"/>
+      <c r="D11" s="158"/>
+      <c r="E11" s="159"/>
+      <c r="F11" s="157" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="159"/>
-      <c r="H11" s="159"/>
-      <c r="I11" s="159"/>
+      <c r="G11" s="158"/>
+      <c r="H11" s="158"/>
+      <c r="I11" s="158"/>
       <c r="J11" s="43"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
@@ -2122,18 +2125,18 @@
       <c r="Z11" s="7"/>
     </row>
     <row r="12" spans="2:30" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="161" t="s">
+      <c r="B12" s="160" t="s">
         <v>93</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
-      <c r="E12" s="157"/>
-      <c r="F12" s="161" t="s">
+      <c r="E12" s="156"/>
+      <c r="F12" s="160" t="s">
         <v>93</v>
       </c>
       <c r="G12" s="4"/>
-      <c r="H12" s="164"/>
-      <c r="I12" s="164"/>
+      <c r="H12" s="163"/>
+      <c r="I12" s="163"/>
       <c r="J12" s="43"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
@@ -2149,18 +2152,18 @@
       <c r="Z12" s="7"/>
     </row>
     <row r="13" spans="2:30" ht="27.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="197" t="s">
+      <c r="B13" s="201" t="s">
         <v>94</v>
       </c>
-      <c r="C13" s="198"/>
-      <c r="D13" s="198"/>
-      <c r="E13" s="199"/>
-      <c r="F13" s="197" t="s">
+      <c r="C13" s="202"/>
+      <c r="D13" s="202"/>
+      <c r="E13" s="203"/>
+      <c r="F13" s="201" t="s">
         <v>94</v>
       </c>
-      <c r="G13" s="198"/>
-      <c r="H13" s="198"/>
-      <c r="I13" s="198"/>
+      <c r="G13" s="202"/>
+      <c r="H13" s="202"/>
+      <c r="I13" s="202"/>
       <c r="J13" s="19"/>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
@@ -2178,18 +2181,18 @@
       <c r="AA13" s="7"/>
     </row>
     <row r="14" spans="2:30" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="197" t="s">
+      <c r="B14" s="201" t="s">
         <v>95</v>
       </c>
-      <c r="C14" s="198"/>
-      <c r="D14" s="198"/>
-      <c r="E14" s="199"/>
-      <c r="F14" s="197" t="s">
+      <c r="C14" s="202"/>
+      <c r="D14" s="202"/>
+      <c r="E14" s="203"/>
+      <c r="F14" s="201" t="s">
         <v>96</v>
       </c>
-      <c r="G14" s="198"/>
-      <c r="H14" s="198"/>
-      <c r="I14" s="198"/>
+      <c r="G14" s="202"/>
+      <c r="H14" s="202"/>
+      <c r="I14" s="202"/>
       <c r="J14" s="19"/>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
@@ -2207,18 +2210,18 @@
       <c r="AA14" s="7"/>
     </row>
     <row r="15" spans="2:30" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="197" t="s">
+      <c r="B15" s="201" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="198"/>
-      <c r="D15" s="198"/>
-      <c r="E15" s="199"/>
-      <c r="F15" s="197" t="s">
+      <c r="C15" s="202"/>
+      <c r="D15" s="202"/>
+      <c r="E15" s="203"/>
+      <c r="F15" s="201" t="s">
         <v>8</v>
       </c>
-      <c r="G15" s="198"/>
-      <c r="H15" s="198"/>
-      <c r="I15" s="198"/>
+      <c r="G15" s="202"/>
+      <c r="H15" s="202"/>
+      <c r="I15" s="202"/>
       <c r="J15" s="19"/>
       <c r="N15" s="7"/>
       <c r="O15" s="7"/>
@@ -2236,18 +2239,18 @@
       <c r="AA15" s="7"/>
     </row>
     <row r="16" spans="2:30" ht="1.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="161" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="162"/>
-      <c r="D16" s="162"/>
-      <c r="E16" s="156"/>
-      <c r="F16" s="161" t="s">
-        <v>17</v>
-      </c>
-      <c r="G16" s="162"/>
-      <c r="H16" s="162"/>
-      <c r="I16" s="163"/>
+      <c r="B16" s="160" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="161"/>
+      <c r="D16" s="161"/>
+      <c r="E16" s="155"/>
+      <c r="F16" s="160" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="161"/>
+      <c r="H16" s="161"/>
+      <c r="I16" s="162"/>
       <c r="J16" s="19"/>
       <c r="N16" s="7"/>
       <c r="O16" s="7"/>
@@ -2265,18 +2268,18 @@
       <c r="AA16" s="7"/>
     </row>
     <row r="17" spans="2:30" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="209" t="s">
+      <c r="B17" s="213" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="210"/>
-      <c r="D17" s="210"/>
-      <c r="E17" s="211"/>
-      <c r="F17" s="209" t="s">
+      <c r="C17" s="214"/>
+      <c r="D17" s="214"/>
+      <c r="E17" s="215"/>
+      <c r="F17" s="213" t="s">
         <v>34</v>
       </c>
-      <c r="G17" s="210"/>
-      <c r="H17" s="210"/>
-      <c r="I17" s="210"/>
+      <c r="G17" s="214"/>
+      <c r="H17" s="214"/>
+      <c r="I17" s="214"/>
       <c r="J17" s="19"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
@@ -2294,18 +2297,18 @@
       <c r="AA17" s="7"/>
     </row>
     <row r="18" spans="2:30" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="212" t="s">
+      <c r="B18" s="216" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="213"/>
+      <c r="C18" s="217"/>
       <c r="D18" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="213" t="s">
+      <c r="E18" s="217" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="213"/>
-      <c r="G18" s="213"/>
+      <c r="F18" s="217"/>
+      <c r="G18" s="217"/>
       <c r="H18" s="20" t="s">
         <v>115</v>
       </c>
@@ -2329,22 +2332,22 @@
       <c r="AA18" s="7"/>
     </row>
     <row r="19" spans="2:30" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="214" t="s">
+      <c r="B19" s="218" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="215"/>
+      <c r="C19" s="219"/>
       <c r="D19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="216" t="s">
+      <c r="E19" s="220" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="217"/>
-      <c r="G19" s="217"/>
-      <c r="H19" s="187" t="s">
+      <c r="F19" s="221"/>
+      <c r="G19" s="221"/>
+      <c r="H19" s="186" t="s">
         <v>12</v>
       </c>
-      <c r="I19" s="188" t="s">
+      <c r="I19" s="187" t="s">
         <v>13</v>
       </c>
       <c r="J19" s="2"/>
@@ -2367,15 +2370,15 @@
       <c r="AD19" s="7"/>
     </row>
     <row r="20" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="183"/>
-      <c r="C20" s="184"/>
-      <c r="D20" s="184"/>
-      <c r="E20" s="185"/>
-      <c r="F20" s="190"/>
-      <c r="G20" s="186"/>
-      <c r="H20" s="187"/>
-      <c r="I20" s="191"/>
-      <c r="J20" s="196"/>
+      <c r="B20" s="182"/>
+      <c r="C20" s="183"/>
+      <c r="D20" s="183"/>
+      <c r="E20" s="184"/>
+      <c r="F20" s="189"/>
+      <c r="G20" s="185"/>
+      <c r="H20" s="186"/>
+      <c r="I20" s="190"/>
+      <c r="J20" s="195"/>
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
@@ -2395,15 +2398,15 @@
       <c r="AD20" s="7"/>
     </row>
     <row r="21" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="183"/>
-      <c r="C21" s="184"/>
-      <c r="D21" s="184"/>
-      <c r="E21" s="185"/>
-      <c r="F21" s="189"/>
-      <c r="G21" s="185"/>
-      <c r="H21" s="184"/>
-      <c r="I21" s="193"/>
-      <c r="J21" s="196"/>
+      <c r="B21" s="182"/>
+      <c r="C21" s="183"/>
+      <c r="D21" s="183"/>
+      <c r="E21" s="184"/>
+      <c r="F21" s="188"/>
+      <c r="G21" s="184"/>
+      <c r="H21" s="183"/>
+      <c r="I21" s="192"/>
+      <c r="J21" s="195"/>
       <c r="N21" s="7"/>
       <c r="O21" s="7"/>
       <c r="P21" s="7"/>
@@ -2423,15 +2426,15 @@
       <c r="AD21" s="7"/>
     </row>
     <row r="22" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="183"/>
-      <c r="C22" s="184"/>
-      <c r="D22" s="184"/>
-      <c r="E22" s="185"/>
-      <c r="F22" s="189"/>
-      <c r="G22" s="185"/>
-      <c r="H22" s="184"/>
-      <c r="I22" s="193"/>
-      <c r="J22" s="196"/>
+      <c r="B22" s="182"/>
+      <c r="C22" s="183"/>
+      <c r="D22" s="183"/>
+      <c r="E22" s="184"/>
+      <c r="F22" s="188"/>
+      <c r="G22" s="184"/>
+      <c r="H22" s="183"/>
+      <c r="I22" s="192"/>
+      <c r="J22" s="195"/>
       <c r="N22" s="7"/>
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
@@ -2451,15 +2454,15 @@
       <c r="AD22" s="7"/>
     </row>
     <row r="23" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="183"/>
-      <c r="C23" s="184"/>
-      <c r="D23" s="184"/>
-      <c r="E23" s="185"/>
-      <c r="F23" s="189"/>
-      <c r="G23" s="185"/>
-      <c r="H23" s="184"/>
-      <c r="I23" s="193"/>
-      <c r="J23" s="196"/>
+      <c r="B23" s="182"/>
+      <c r="C23" s="183"/>
+      <c r="D23" s="183"/>
+      <c r="E23" s="184"/>
+      <c r="F23" s="188"/>
+      <c r="G23" s="184"/>
+      <c r="H23" s="183"/>
+      <c r="I23" s="192"/>
+      <c r="J23" s="195"/>
       <c r="N23" s="7"/>
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
@@ -2479,15 +2482,15 @@
       <c r="AD23" s="7"/>
     </row>
     <row r="24" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="183"/>
-      <c r="C24" s="184"/>
-      <c r="D24" s="184"/>
-      <c r="E24" s="185"/>
-      <c r="F24" s="189"/>
-      <c r="G24" s="185"/>
-      <c r="H24" s="184"/>
-      <c r="I24" s="193"/>
-      <c r="J24" s="196"/>
+      <c r="B24" s="182"/>
+      <c r="C24" s="183"/>
+      <c r="D24" s="183"/>
+      <c r="E24" s="184"/>
+      <c r="F24" s="188"/>
+      <c r="G24" s="184"/>
+      <c r="H24" s="183"/>
+      <c r="I24" s="192"/>
+      <c r="J24" s="195"/>
       <c r="N24" s="7"/>
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
@@ -2507,15 +2510,15 @@
       <c r="AD24" s="7"/>
     </row>
     <row r="25" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="183"/>
-      <c r="C25" s="184"/>
-      <c r="D25" s="184"/>
-      <c r="E25" s="185"/>
-      <c r="F25" s="189"/>
-      <c r="G25" s="185"/>
-      <c r="H25" s="184"/>
-      <c r="I25" s="193"/>
-      <c r="J25" s="196"/>
+      <c r="B25" s="182"/>
+      <c r="C25" s="183"/>
+      <c r="D25" s="183"/>
+      <c r="E25" s="184"/>
+      <c r="F25" s="188"/>
+      <c r="G25" s="184"/>
+      <c r="H25" s="183"/>
+      <c r="I25" s="192"/>
+      <c r="J25" s="195"/>
       <c r="N25" s="7"/>
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
@@ -2535,15 +2538,15 @@
       <c r="AD25" s="7"/>
     </row>
     <row r="26" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="183"/>
-      <c r="C26" s="184"/>
-      <c r="D26" s="184"/>
-      <c r="E26" s="185"/>
-      <c r="F26" s="189"/>
-      <c r="G26" s="185"/>
-      <c r="H26" s="184"/>
-      <c r="I26" s="193"/>
-      <c r="J26" s="196"/>
+      <c r="B26" s="182"/>
+      <c r="C26" s="183"/>
+      <c r="D26" s="183"/>
+      <c r="E26" s="184"/>
+      <c r="F26" s="188"/>
+      <c r="G26" s="184"/>
+      <c r="H26" s="183"/>
+      <c r="I26" s="192"/>
+      <c r="J26" s="195"/>
       <c r="N26" s="7"/>
       <c r="O26" s="7"/>
       <c r="P26" s="7"/>
@@ -2563,14 +2566,14 @@
       <c r="AD26" s="7"/>
     </row>
     <row r="27" spans="2:30" ht="0.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="183"/>
-      <c r="C27" s="184"/>
-      <c r="D27" s="184"/>
-      <c r="E27" s="185"/>
-      <c r="F27" s="189"/>
-      <c r="G27" s="185"/>
-      <c r="H27" s="184"/>
-      <c r="I27" s="193"/>
+      <c r="B27" s="182"/>
+      <c r="C27" s="183"/>
+      <c r="D27" s="183"/>
+      <c r="E27" s="184"/>
+      <c r="F27" s="188"/>
+      <c r="G27" s="184"/>
+      <c r="H27" s="183"/>
+      <c r="I27" s="192"/>
       <c r="J27" s="2"/>
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
@@ -2591,18 +2594,18 @@
       <c r="AD27" s="7"/>
     </row>
     <row r="28" spans="2:30" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="150" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="166"/>
-      <c r="D28" s="166"/>
-      <c r="E28" s="167"/>
-      <c r="F28" s="150" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" s="167"/>
-      <c r="H28" s="166"/>
-      <c r="I28" s="192"/>
+      <c r="B28" s="149" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="165"/>
+      <c r="D28" s="165"/>
+      <c r="E28" s="166"/>
+      <c r="F28" s="149" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" s="166"/>
+      <c r="H28" s="165"/>
+      <c r="I28" s="191"/>
       <c r="J28" s="2"/>
       <c r="N28" s="7"/>
       <c r="O28" s="7"/>
@@ -2623,19 +2626,19 @@
       <c r="AD28" s="7"/>
     </row>
     <row r="29" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="189" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="184"/>
-      <c r="D29" s="184"/>
-      <c r="E29" s="185"/>
-      <c r="F29" s="189" t="s">
-        <v>17</v>
-      </c>
-      <c r="G29" s="185"/>
-      <c r="H29" s="184"/>
-      <c r="I29" s="193"/>
-      <c r="J29" s="168"/>
+      <c r="B29" s="188" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="183"/>
+      <c r="D29" s="183"/>
+      <c r="E29" s="184"/>
+      <c r="F29" s="188" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="184"/>
+      <c r="H29" s="183"/>
+      <c r="I29" s="192"/>
+      <c r="J29" s="167"/>
       <c r="N29" s="7"/>
       <c r="O29" s="7"/>
       <c r="P29" s="7"/>
@@ -2655,19 +2658,19 @@
       <c r="AD29" s="7"/>
     </row>
     <row r="30" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="171" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="173"/>
-      <c r="D30" s="173"/>
-      <c r="E30" s="173"/>
-      <c r="F30" s="171" t="s">
-        <v>17</v>
-      </c>
-      <c r="G30" s="173"/>
-      <c r="H30" s="172"/>
-      <c r="I30" s="174"/>
-      <c r="J30" s="168"/>
+      <c r="B30" s="170" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="172"/>
+      <c r="D30" s="172"/>
+      <c r="E30" s="172"/>
+      <c r="F30" s="170" t="s">
+        <v>17</v>
+      </c>
+      <c r="G30" s="172"/>
+      <c r="H30" s="171"/>
+      <c r="I30" s="173"/>
+      <c r="J30" s="167"/>
       <c r="N30" s="7"/>
       <c r="O30" s="7"/>
       <c r="P30" s="7"/>
@@ -2687,19 +2690,19 @@
       <c r="AD30" s="7"/>
     </row>
     <row r="31" spans="2:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="171" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="173"/>
-      <c r="D31" s="173"/>
-      <c r="E31" s="173"/>
-      <c r="F31" s="171" t="s">
-        <v>17</v>
-      </c>
-      <c r="G31" s="173"/>
-      <c r="H31" s="172"/>
-      <c r="I31" s="174"/>
-      <c r="J31" s="168"/>
+      <c r="B31" s="170" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="172"/>
+      <c r="D31" s="172"/>
+      <c r="E31" s="172"/>
+      <c r="F31" s="170" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" s="172"/>
+      <c r="H31" s="171"/>
+      <c r="I31" s="173"/>
+      <c r="J31" s="167"/>
       <c r="N31" s="7"/>
       <c r="O31" s="7"/>
       <c r="P31" s="7"/>
@@ -2724,14 +2727,14 @@
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
-      <c r="E32" s="167"/>
-      <c r="F32" s="158" t="s">
+      <c r="E32" s="166"/>
+      <c r="F32" s="157" t="s">
         <v>17</v>
       </c>
       <c r="G32" s="5"/>
-      <c r="H32" s="181"/>
-      <c r="I32" s="182"/>
-      <c r="J32" s="168"/>
+      <c r="H32" s="180"/>
+      <c r="I32" s="181"/>
+      <c r="J32" s="167"/>
       <c r="N32" s="7"/>
       <c r="O32" s="7"/>
       <c r="P32" s="7"/>
@@ -2751,19 +2754,19 @@
       <c r="AD32" s="7"/>
     </row>
     <row r="33" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="171" t="s">
-        <v>17</v>
-      </c>
-      <c r="C33" s="175"/>
-      <c r="D33" s="175"/>
-      <c r="E33" s="173"/>
-      <c r="F33" s="171" t="s">
-        <v>17</v>
-      </c>
-      <c r="G33" s="176"/>
-      <c r="H33" s="177"/>
-      <c r="I33" s="178"/>
-      <c r="J33" s="168"/>
+      <c r="B33" s="170" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" s="174"/>
+      <c r="D33" s="174"/>
+      <c r="E33" s="172"/>
+      <c r="F33" s="170" t="s">
+        <v>17</v>
+      </c>
+      <c r="G33" s="175"/>
+      <c r="H33" s="176"/>
+      <c r="I33" s="177"/>
+      <c r="J33" s="167"/>
       <c r="N33" s="7"/>
       <c r="O33" s="7"/>
       <c r="P33" s="7"/>
@@ -2795,21 +2798,21 @@
       <c r="G34" s="17"/>
       <c r="H34" s="17"/>
       <c r="I34" s="18"/>
-      <c r="J34" s="154"/>
+      <c r="J34" s="153"/>
     </row>
     <row r="35" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="169" t="s">
+      <c r="B35" s="168" t="s">
         <v>17</v>
       </c>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="12"/>
-      <c r="F35" s="158" t="s">
+      <c r="F35" s="157" t="s">
         <v>17</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="12"/>
-      <c r="I35" s="155"/>
+      <c r="I35" s="154"/>
       <c r="J35" s="13"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
@@ -2830,18 +2833,18 @@
       <c r="AD35" s="7"/>
     </row>
     <row r="36" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="197" t="s">
-        <v>17</v>
-      </c>
-      <c r="C36" s="198"/>
-      <c r="D36" s="198"/>
-      <c r="E36" s="198"/>
-      <c r="F36" s="197" t="s">
-        <v>17</v>
-      </c>
-      <c r="G36" s="198"/>
-      <c r="H36" s="198"/>
-      <c r="I36" s="199"/>
+      <c r="B36" s="201" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="202"/>
+      <c r="D36" s="202"/>
+      <c r="E36" s="202"/>
+      <c r="F36" s="201" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" s="202"/>
+      <c r="H36" s="202"/>
+      <c r="I36" s="203"/>
       <c r="J36" s="13"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
@@ -2926,48 +2929,48 @@
       <c r="AD38" s="7"/>
     </row>
     <row r="39" spans="1:30" s="27" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="204" t="s">
+      <c r="B39" s="208" t="s">
         <v>80</v>
       </c>
-      <c r="C39" s="205"/>
-      <c r="D39" s="205"/>
-      <c r="E39" s="205"/>
-      <c r="F39" s="204" t="s">
+      <c r="C39" s="209"/>
+      <c r="D39" s="209"/>
+      <c r="E39" s="209"/>
+      <c r="F39" s="208" t="s">
         <v>80</v>
       </c>
-      <c r="G39" s="205"/>
-      <c r="H39" s="205"/>
-      <c r="I39" s="206"/>
-      <c r="J39" s="154"/>
+      <c r="G39" s="209"/>
+      <c r="H39" s="209"/>
+      <c r="I39" s="210"/>
+      <c r="J39" s="153"/>
     </row>
     <row r="40" spans="1:30" s="27" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="207" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="208"/>
-      <c r="D40" s="208"/>
-      <c r="E40" s="208"/>
-      <c r="F40" s="197" t="s">
-        <v>17</v>
-      </c>
-      <c r="G40" s="198"/>
-      <c r="H40" s="198"/>
-      <c r="I40" s="199"/>
-      <c r="J40" s="154"/>
+      <c r="B40" s="211" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="212"/>
+      <c r="D40" s="212"/>
+      <c r="E40" s="212"/>
+      <c r="F40" s="201" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="202"/>
+      <c r="H40" s="202"/>
+      <c r="I40" s="203"/>
+      <c r="J40" s="153"/>
     </row>
     <row r="41" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="169" t="s">
+      <c r="B41" s="168" t="s">
         <v>17</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="12"/>
-      <c r="F41" s="158" t="s">
-        <v>17</v>
-      </c>
-      <c r="G41" s="159"/>
-      <c r="H41" s="179"/>
-      <c r="I41" s="180"/>
+      <c r="F41" s="157" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" s="158"/>
+      <c r="H41" s="178"/>
+      <c r="I41" s="179"/>
       <c r="J41" s="13"/>
       <c r="N41" s="7"/>
       <c r="O41" s="7"/>
@@ -2988,55 +2991,55 @@
       <c r="AD41" s="7"/>
     </row>
     <row r="42" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="197" t="s">
-        <v>17</v>
-      </c>
-      <c r="C42" s="198"/>
-      <c r="D42" s="198"/>
-      <c r="E42" s="198"/>
-      <c r="F42" s="197" t="s">
-        <v>17</v>
-      </c>
-      <c r="G42" s="198"/>
-      <c r="H42" s="198"/>
-      <c r="I42" s="199"/>
+      <c r="B42" s="201" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="202"/>
+      <c r="D42" s="202"/>
+      <c r="E42" s="202"/>
+      <c r="F42" s="201" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" s="202"/>
+      <c r="H42" s="202"/>
+      <c r="I42" s="203"/>
       <c r="J42" s="6"/>
     </row>
     <row r="43" spans="1:30" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="194" t="s">
+      <c r="B43" s="193" t="s">
         <v>14</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="12"/>
-      <c r="F43" s="195" t="s">
+      <c r="F43" s="194" t="s">
         <v>15</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
-      <c r="I43" s="157"/>
+      <c r="I43" s="156"/>
       <c r="J43" s="6"/>
     </row>
     <row r="44" spans="1:30" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="170"/>
-      <c r="B44" s="169"/>
+      <c r="A44" s="169"/>
+      <c r="B44" s="168"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
-      <c r="F44" s="169"/>
+      <c r="F44" s="168"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
       <c r="I44" s="42"/>
       <c r="J44" s="6"/>
     </row>
     <row r="45" spans="1:30" ht="19.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="158" t="s">
+      <c r="B45" s="157" t="s">
         <v>22</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="12"/>
-      <c r="F45" s="158" t="s">
+      <c r="F45" s="157" t="s">
         <v>27</v>
       </c>
       <c r="G45" s="5"/>
@@ -3045,18 +3048,18 @@
       <c r="J45" s="6"/>
     </row>
     <row r="46" spans="1:30" s="27" customFormat="1" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="200" t="s">
+      <c r="B46" s="204" t="s">
         <v>93</v>
       </c>
-      <c r="C46" s="201"/>
-      <c r="D46" s="201"/>
-      <c r="E46" s="201"/>
-      <c r="F46" s="200" t="s">
+      <c r="C46" s="205"/>
+      <c r="D46" s="205"/>
+      <c r="E46" s="205"/>
+      <c r="F46" s="204" t="s">
         <v>97</v>
       </c>
-      <c r="G46" s="201"/>
-      <c r="H46" s="201"/>
-      <c r="I46" s="202"/>
+      <c r="G46" s="205"/>
+      <c r="H46" s="205"/>
+      <c r="I46" s="206"/>
       <c r="J46" s="26"/>
       <c r="N46" s="28"/>
       <c r="O46" s="28"/>
@@ -3077,103 +3080,103 @@
       <c r="AD46" s="28"/>
     </row>
     <row r="47" spans="1:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="197" t="s">
+      <c r="B47" s="201" t="s">
         <v>94</v>
       </c>
-      <c r="C47" s="198"/>
-      <c r="D47" s="198"/>
-      <c r="E47" s="198"/>
-      <c r="F47" s="197" t="s">
+      <c r="C47" s="202"/>
+      <c r="D47" s="202"/>
+      <c r="E47" s="202"/>
+      <c r="F47" s="201" t="s">
         <v>98</v>
       </c>
-      <c r="G47" s="198"/>
-      <c r="H47" s="198"/>
-      <c r="I47" s="199"/>
+      <c r="G47" s="202"/>
+      <c r="H47" s="202"/>
+      <c r="I47" s="203"/>
       <c r="J47" s="16"/>
     </row>
     <row r="48" spans="1:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="197" t="s">
+      <c r="B48" s="201" t="s">
         <v>100</v>
       </c>
-      <c r="C48" s="198"/>
-      <c r="D48" s="198"/>
-      <c r="E48" s="199"/>
-      <c r="F48" s="197" t="s">
+      <c r="C48" s="202"/>
+      <c r="D48" s="202"/>
+      <c r="E48" s="203"/>
+      <c r="F48" s="201" t="s">
         <v>99</v>
       </c>
-      <c r="G48" s="198"/>
-      <c r="H48" s="198"/>
-      <c r="I48" s="198"/>
+      <c r="G48" s="202"/>
+      <c r="H48" s="202"/>
+      <c r="I48" s="202"/>
       <c r="J48" s="16"/>
     </row>
     <row r="49" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="197" t="s">
+      <c r="B49" s="201" t="s">
         <v>101</v>
       </c>
-      <c r="C49" s="198"/>
-      <c r="D49" s="198"/>
-      <c r="E49" s="199"/>
-      <c r="F49" s="197" t="s">
+      <c r="C49" s="202"/>
+      <c r="D49" s="202"/>
+      <c r="E49" s="203"/>
+      <c r="F49" s="201" t="s">
         <v>102</v>
       </c>
-      <c r="G49" s="198"/>
-      <c r="H49" s="198"/>
-      <c r="I49" s="198"/>
+      <c r="G49" s="202"/>
+      <c r="H49" s="202"/>
+      <c r="I49" s="202"/>
       <c r="J49" s="16"/>
     </row>
     <row r="50" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="197" t="s">
+      <c r="B50" s="201" t="s">
         <v>103</v>
       </c>
-      <c r="C50" s="198"/>
-      <c r="D50" s="198"/>
-      <c r="E50" s="199"/>
-      <c r="F50" s="197" t="s">
+      <c r="C50" s="202"/>
+      <c r="D50" s="202"/>
+      <c r="E50" s="203"/>
+      <c r="F50" s="201" t="s">
         <v>103</v>
       </c>
-      <c r="G50" s="198"/>
-      <c r="H50" s="198"/>
-      <c r="I50" s="198"/>
+      <c r="G50" s="202"/>
+      <c r="H50" s="202"/>
+      <c r="I50" s="202"/>
       <c r="J50" s="16"/>
     </row>
     <row r="51" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="197" t="s">
+      <c r="B51" s="201" t="s">
         <v>104</v>
       </c>
-      <c r="C51" s="198"/>
-      <c r="D51" s="198"/>
-      <c r="E51" s="199"/>
-      <c r="F51" s="197" t="s">
+      <c r="C51" s="202"/>
+      <c r="D51" s="202"/>
+      <c r="E51" s="203"/>
+      <c r="F51" s="201" t="s">
         <v>105</v>
       </c>
-      <c r="G51" s="198"/>
-      <c r="H51" s="198"/>
-      <c r="I51" s="198"/>
+      <c r="G51" s="202"/>
+      <c r="H51" s="202"/>
+      <c r="I51" s="202"/>
       <c r="J51" s="16"/>
     </row>
     <row r="52" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="197" t="s">
+      <c r="B52" s="201" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="198"/>
-      <c r="D52" s="198"/>
-      <c r="E52" s="199"/>
-      <c r="F52" s="197" t="s">
+      <c r="C52" s="202"/>
+      <c r="D52" s="202"/>
+      <c r="E52" s="203"/>
+      <c r="F52" s="201" t="s">
         <v>107</v>
       </c>
-      <c r="G52" s="198"/>
-      <c r="H52" s="198"/>
-      <c r="I52" s="198"/>
+      <c r="G52" s="202"/>
+      <c r="H52" s="202"/>
+      <c r="I52" s="202"/>
       <c r="J52" s="16"/>
     </row>
     <row r="53" spans="2:30" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="169" t="s">
+      <c r="B53" s="168" t="s">
         <v>28</v>
       </c>
       <c r="C53" s="12"/>
       <c r="D53" s="12"/>
-      <c r="E53" s="155"/>
-      <c r="F53" s="169" t="s">
+      <c r="E53" s="154"/>
+      <c r="F53" s="168" t="s">
         <v>29</v>
       </c>
       <c r="G53" s="17"/>
@@ -3182,18 +3185,18 @@
       <c r="J53" s="16"/>
     </row>
     <row r="54" spans="2:30" s="27" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="200" t="s">
+      <c r="B54" s="204" t="s">
         <v>93</v>
       </c>
-      <c r="C54" s="201"/>
-      <c r="D54" s="201"/>
-      <c r="E54" s="202"/>
-      <c r="F54" s="200" t="s">
+      <c r="C54" s="205"/>
+      <c r="D54" s="205"/>
+      <c r="E54" s="206"/>
+      <c r="F54" s="204" t="s">
         <v>93</v>
       </c>
-      <c r="G54" s="203"/>
-      <c r="H54" s="203"/>
-      <c r="I54" s="203"/>
+      <c r="G54" s="207"/>
+      <c r="H54" s="207"/>
+      <c r="I54" s="207"/>
       <c r="J54" s="26"/>
       <c r="N54" s="28"/>
       <c r="O54" s="28"/>
@@ -3214,18 +3217,18 @@
       <c r="AD54" s="28"/>
     </row>
     <row r="55" spans="2:30" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="197" t="s">
+      <c r="B55" s="201" t="s">
         <v>108</v>
       </c>
-      <c r="C55" s="198"/>
-      <c r="D55" s="198"/>
-      <c r="E55" s="199"/>
-      <c r="F55" s="197" t="s">
+      <c r="C55" s="202"/>
+      <c r="D55" s="202"/>
+      <c r="E55" s="203"/>
+      <c r="F55" s="201" t="s">
         <v>108</v>
       </c>
-      <c r="G55" s="198"/>
-      <c r="H55" s="198"/>
-      <c r="I55" s="198"/>
+      <c r="G55" s="202"/>
+      <c r="H55" s="202"/>
+      <c r="I55" s="202"/>
       <c r="J55" s="16"/>
     </row>
     <row r="56" spans="2:30" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3285,18 +3288,18 @@
       <c r="J59" s="16"/>
     </row>
     <row r="60" spans="2:30" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="197" t="s">
+      <c r="B60" s="201" t="s">
         <v>101</v>
       </c>
-      <c r="C60" s="198"/>
-      <c r="D60" s="198"/>
-      <c r="E60" s="199"/>
-      <c r="F60" s="197" t="s">
+      <c r="C60" s="202"/>
+      <c r="D60" s="202"/>
+      <c r="E60" s="203"/>
+      <c r="F60" s="201" t="s">
         <v>101</v>
       </c>
-      <c r="G60" s="198"/>
-      <c r="H60" s="198"/>
-      <c r="I60" s="199"/>
+      <c r="G60" s="202"/>
+      <c r="H60" s="202"/>
+      <c r="I60" s="203"/>
       <c r="J60" s="16"/>
     </row>
     <row r="61" spans="2:30" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3593,7 +3596,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.35433070866141736" bottom="0.15748031496062992" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="76" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="75" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3607,7 +3610,7 @@
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" customWidth="1"/>
     <col min="5" max="5" width="8.42578125" customWidth="1"/>
@@ -3625,89 +3628,89 @@
   <sheetData>
     <row r="1" spans="1:14" ht="3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="45"/>
-      <c r="G1" s="142" t="s">
+      <c r="G1" s="141" t="s">
         <v>17</v>
       </c>
       <c r="N1" s="47"/>
     </row>
     <row r="2" spans="1:14" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="76"/>
-      <c r="B2" s="104" t="s">
+      <c r="B2" s="103" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="107" t="s">
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="106" t="s">
         <v>76</v>
       </c>
-      <c r="I2" s="104"/>
-      <c r="J2" s="104"/>
-      <c r="K2" s="104"/>
-      <c r="L2" s="104"/>
-      <c r="M2" s="104"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
       <c r="N2" s="47"/>
     </row>
     <row r="3" spans="1:14" ht="33.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="76"/>
-      <c r="B3" s="105" t="s">
+      <c r="B3" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="105"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="106"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="108" t="s">
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="105"/>
+      <c r="G3" s="105"/>
+      <c r="H3" s="107" t="s">
         <v>74</v>
       </c>
-      <c r="I3" s="105"/>
-      <c r="J3" s="105"/>
-      <c r="K3" s="105"/>
-      <c r="L3" s="105"/>
-      <c r="M3" s="105"/>
+      <c r="I3" s="104"/>
+      <c r="J3" s="104"/>
+      <c r="K3" s="104"/>
+      <c r="L3" s="104"/>
+      <c r="M3" s="104"/>
       <c r="N3" s="47"/>
     </row>
     <row r="4" spans="1:14" s="73" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75"/>
-      <c r="B4" s="105" t="s">
+      <c r="B4" s="104" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="105"/>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="105"/>
-      <c r="H4" s="108" t="s">
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="107" t="s">
         <v>72</v>
       </c>
-      <c r="I4" s="105"/>
-      <c r="J4" s="105"/>
-      <c r="K4" s="105"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="105"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="104"/>
+      <c r="M4" s="104"/>
       <c r="N4" s="71"/>
     </row>
     <row r="5" spans="1:14" s="73" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="74"/>
-      <c r="B5" s="105" t="s">
+      <c r="B5" s="104" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="105"/>
-      <c r="D5" s="105"/>
-      <c r="E5" s="105"/>
-      <c r="F5" s="105"/>
-      <c r="G5" s="105"/>
-      <c r="H5" s="108" t="s">
+      <c r="C5" s="104"/>
+      <c r="D5" s="104"/>
+      <c r="E5" s="104"/>
+      <c r="F5" s="104"/>
+      <c r="G5" s="104"/>
+      <c r="H5" s="107" t="s">
         <v>70</v>
       </c>
-      <c r="I5" s="105"/>
-      <c r="J5" s="105"/>
-      <c r="K5" s="105"/>
-      <c r="L5" s="105"/>
-      <c r="M5" s="105"/>
+      <c r="I5" s="104"/>
+      <c r="J5" s="104"/>
+      <c r="K5" s="104"/>
+      <c r="L5" s="104"/>
+      <c r="M5" s="104"/>
       <c r="N5" s="71"/>
     </row>
     <row r="6" spans="1:14" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -3735,11 +3738,11 @@
       <c r="B7" s="98" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="109"/>
-      <c r="D7" s="109"/>
-      <c r="E7" s="109"/>
-      <c r="F7" s="109"/>
-      <c r="G7" s="109"/>
+      <c r="C7" s="108"/>
+      <c r="D7" s="108"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
       <c r="H7" s="85" t="s">
         <v>2</v>
       </c>
@@ -3752,14 +3755,14 @@
     </row>
     <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="45"/>
-      <c r="B8" s="110" t="s">
+      <c r="B8" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="110"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="110"/>
-      <c r="F8" s="110"/>
-      <c r="G8" s="110"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="109"/>
+      <c r="E8" s="109"/>
+      <c r="F8" s="109"/>
+      <c r="G8" s="109"/>
       <c r="H8" s="87" t="s">
         <v>4</v>
       </c>
@@ -3772,14 +3775,14 @@
     </row>
     <row r="9" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="45"/>
-      <c r="B9" s="111" t="s">
+      <c r="B9" s="110" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="111"/>
-      <c r="D9" s="111"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="111"/>
-      <c r="G9" s="111"/>
+      <c r="C9" s="110"/>
+      <c r="D9" s="110"/>
+      <c r="E9" s="110"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
       <c r="H9" s="89" t="s">
         <v>78</v>
       </c>
@@ -3819,8 +3822,8 @@
       <c r="D11" s="88"/>
       <c r="E11" s="88"/>
       <c r="F11" s="88"/>
-      <c r="G11" s="103"/>
-      <c r="H11" s="140" t="s">
+      <c r="G11" s="102"/>
+      <c r="H11" s="139" t="s">
         <v>6</v>
       </c>
       <c r="I11" s="88"/>
@@ -3832,14 +3835,14 @@
     </row>
     <row r="12" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="45"/>
-      <c r="B12" s="111" t="s">
+      <c r="B12" s="110" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="111"/>
-      <c r="D12" s="111"/>
-      <c r="E12" s="111"/>
-      <c r="F12" s="111"/>
-      <c r="G12" s="111"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
       <c r="H12" s="82" t="s">
         <v>67</v>
       </c>
@@ -3872,15 +3875,15 @@
     </row>
     <row r="14" spans="1:14" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="45"/>
-      <c r="B14" s="151" t="s">
+      <c r="B14" s="150" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="152"/>
-      <c r="D14" s="152"/>
-      <c r="E14" s="152"/>
-      <c r="F14" s="152"/>
-      <c r="G14" s="103"/>
-      <c r="H14" s="140" t="s">
+      <c r="C14" s="151"/>
+      <c r="D14" s="151"/>
+      <c r="E14" s="151"/>
+      <c r="F14" s="151"/>
+      <c r="G14" s="102"/>
+      <c r="H14" s="139" t="s">
         <v>6</v>
       </c>
       <c r="I14" s="88"/>
@@ -3892,10 +3895,10 @@
     </row>
     <row r="15" spans="1:14" ht="32.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="72"/>
-      <c r="B15" s="230" t="s">
+      <c r="B15" s="199" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="231"/>
+      <c r="C15" s="200"/>
       <c r="D15" s="90" t="s">
         <v>56</v>
       </c>
@@ -3908,14 +3911,14 @@
         <v>58</v>
       </c>
       <c r="I15" s="90"/>
-      <c r="J15" s="112" t="s">
+      <c r="J15" s="111" t="s">
         <v>56</v>
       </c>
-      <c r="K15" s="112"/>
-      <c r="L15" s="136" t="s">
+      <c r="K15" s="111"/>
+      <c r="L15" s="135" t="s">
         <v>57</v>
       </c>
-      <c r="M15" s="136"/>
+      <c r="M15" s="135"/>
       <c r="N15" s="47"/>
     </row>
     <row r="16" spans="1:14" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
@@ -3928,11 +3931,11 @@
         <v>17</v>
       </c>
       <c r="E16" s="93"/>
-      <c r="F16" s="129" t="s">
+      <c r="F16" s="128" t="s">
         <v>55</v>
       </c>
       <c r="G16" s="93"/>
-      <c r="H16" s="153" t="s">
+      <c r="H16" s="152" t="s">
         <v>17</v>
       </c>
       <c r="I16" s="93"/>
@@ -3940,26 +3943,26 @@
         <v>17</v>
       </c>
       <c r="K16" s="94"/>
-      <c r="L16" s="137" t="s">
+      <c r="L16" s="136" t="s">
         <v>54</v>
       </c>
-      <c r="M16" s="137"/>
+      <c r="M16" s="136"/>
       <c r="N16" s="47"/>
     </row>
     <row r="17" spans="1:29" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45"/>
-      <c r="B17" s="133" t="s">
+      <c r="B17" s="132" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="111"/>
-      <c r="D17" s="130" t="s">
+      <c r="C17" s="110"/>
+      <c r="D17" s="129" t="s">
         <v>65</v>
       </c>
-      <c r="E17" s="115"/>
-      <c r="F17" s="128" t="s">
+      <c r="E17" s="114"/>
+      <c r="F17" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="128"/>
+      <c r="G17" s="127"/>
       <c r="H17" s="89" t="s">
         <v>63</v>
       </c>
@@ -3968,27 +3971,27 @@
         <v>62</v>
       </c>
       <c r="K17" s="84"/>
-      <c r="L17" s="138" t="s">
+      <c r="L17" s="137" t="s">
         <v>61</v>
       </c>
-      <c r="M17" s="139"/>
+      <c r="M17" s="138"/>
       <c r="N17" s="47"/>
     </row>
     <row r="18" spans="1:29" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="45"/>
-      <c r="B18" s="110" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="110"/>
+      <c r="B18" s="109" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="109"/>
       <c r="D18" s="94" t="s">
         <v>17</v>
       </c>
       <c r="E18" s="94"/>
-      <c r="F18" s="141" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" s="129"/>
-      <c r="H18" s="153" t="s">
+      <c r="F18" s="140" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="128"/>
+      <c r="H18" s="152" t="s">
         <v>17</v>
       </c>
       <c r="I18" s="94"/>
@@ -3996,34 +3999,34 @@
         <v>17</v>
       </c>
       <c r="K18" s="94"/>
-      <c r="L18" s="137" t="s">
-        <v>17</v>
-      </c>
-      <c r="M18" s="137"/>
+      <c r="L18" s="196" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="196"/>
       <c r="N18" s="47"/>
     </row>
     <row r="19" spans="1:29" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="45"/>
-      <c r="B19" s="133" t="s">
+      <c r="B19" s="132" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="116"/>
-      <c r="D19" s="116" t="s">
+      <c r="C19" s="115"/>
+      <c r="D19" s="115" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="116"/>
-      <c r="F19" s="116"/>
-      <c r="G19" s="130"/>
-      <c r="H19" s="133" t="s">
+      <c r="E19" s="115"/>
+      <c r="F19" s="115"/>
+      <c r="G19" s="129"/>
+      <c r="H19" s="132" t="s">
         <v>79</v>
       </c>
-      <c r="I19" s="113"/>
-      <c r="J19" s="111" t="s">
+      <c r="I19" s="112"/>
+      <c r="J19" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="K19" s="111"/>
-      <c r="L19" s="111"/>
-      <c r="M19" s="111"/>
+      <c r="K19" s="110"/>
+      <c r="L19" s="110"/>
+      <c r="M19" s="110"/>
       <c r="N19" s="47"/>
     </row>
     <row r="20" spans="1:29" ht="29.85" customHeight="1" x14ac:dyDescent="0.25">
@@ -4032,12 +4035,12 @@
         <v>17</v>
       </c>
       <c r="C20" s="97"/>
-      <c r="D20" s="114" t="s">
-        <v>17</v>
-      </c>
-      <c r="E20" s="114"/>
-      <c r="F20" s="131"/>
-      <c r="G20" s="131"/>
+      <c r="D20" s="113" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="113"/>
+      <c r="F20" s="130"/>
+      <c r="G20" s="130"/>
       <c r="H20" s="85" t="s">
         <v>17</v>
       </c>
@@ -4045,25 +4048,25 @@
       <c r="J20" s="98" t="s">
         <v>17</v>
       </c>
-      <c r="K20" s="99"/>
+      <c r="K20" s="232"/>
       <c r="L20" s="94"/>
       <c r="M20" s="94"/>
       <c r="N20" s="47"/>
     </row>
     <row r="21" spans="1:29" s="69" customFormat="1" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="81"/>
-      <c r="B21" s="100"/>
-      <c r="C21" s="100"/>
-      <c r="D21" s="100"/>
-      <c r="E21" s="100"/>
-      <c r="F21" s="100"/>
-      <c r="G21" s="132"/>
-      <c r="H21" s="134"/>
-      <c r="I21" s="101"/>
-      <c r="J21" s="101"/>
-      <c r="K21" s="101"/>
-      <c r="L21" s="101"/>
-      <c r="M21" s="102"/>
+      <c r="B21" s="99"/>
+      <c r="C21" s="99"/>
+      <c r="D21" s="99"/>
+      <c r="E21" s="99"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="131"/>
+      <c r="H21" s="133"/>
+      <c r="I21" s="100"/>
+      <c r="J21" s="100"/>
+      <c r="K21" s="100"/>
+      <c r="L21" s="100"/>
+      <c r="M21" s="101"/>
       <c r="N21" s="70"/>
       <c r="S21"/>
       <c r="T21"/>
@@ -4082,13 +4085,13 @@
       <c r="B22" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="117" t="s">
+      <c r="C22" s="116" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="117"/>
-      <c r="E22" s="117"/>
-      <c r="F22" s="135"/>
-      <c r="G22" s="117"/>
+      <c r="D22" s="116"/>
+      <c r="E22" s="116"/>
+      <c r="F22" s="134"/>
+      <c r="G22" s="116"/>
       <c r="H22" s="49" t="s">
         <v>48</v>
       </c>
@@ -4098,10 +4101,10 @@
       <c r="J22" s="67" t="s">
         <v>113</v>
       </c>
-      <c r="K22" s="117" t="s">
+      <c r="K22" s="116" t="s">
         <v>114</v>
       </c>
-      <c r="L22" s="117"/>
+      <c r="L22" s="116"/>
       <c r="M22" s="49" t="s">
         <v>46</v>
       </c>
@@ -4109,17 +4112,17 @@
     </row>
     <row r="23" spans="1:29" ht="52.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="45"/>
-      <c r="B23" s="124" t="s">
+      <c r="B23" s="123" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="228" t="s">
+      <c r="C23" s="197" t="s">
         <v>44</v>
       </c>
-      <c r="D23" s="228"/>
-      <c r="E23" s="228"/>
-      <c r="F23" s="228"/>
-      <c r="G23" s="125"/>
-      <c r="H23" s="126" t="s">
+      <c r="D23" s="197"/>
+      <c r="E23" s="197"/>
+      <c r="F23" s="197"/>
+      <c r="G23" s="124"/>
+      <c r="H23" s="125" t="s">
         <v>43</v>
       </c>
       <c r="I23" s="66" t="s">
@@ -4128,10 +4131,10 @@
       <c r="J23" s="65">
         <v>14</v>
       </c>
-      <c r="K23" s="229" t="s">
+      <c r="K23" s="198" t="s">
         <v>42</v>
       </c>
-      <c r="L23" s="229"/>
+      <c r="L23" s="198"/>
       <c r="M23" s="64" t="s">
         <v>39</v>
       </c>
@@ -4139,12 +4142,12 @@
     </row>
     <row r="24" spans="1:29" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="45"/>
-      <c r="C24" s="122"/>
-      <c r="D24" s="122"/>
-      <c r="E24" s="122"/>
-      <c r="F24" s="122"/>
-      <c r="G24" s="122"/>
-      <c r="H24" s="123" t="s">
+      <c r="C24" s="121"/>
+      <c r="D24" s="121"/>
+      <c r="E24" s="121"/>
+      <c r="F24" s="121"/>
+      <c r="G24" s="121"/>
+      <c r="H24" s="122" t="s">
         <v>41</v>
       </c>
       <c r="I24" s="63" t="s">
@@ -4153,10 +4156,10 @@
       <c r="J24" s="62">
         <v>14</v>
       </c>
-      <c r="K24" s="127" t="s">
-        <v>17</v>
-      </c>
-      <c r="L24" s="127"/>
+      <c r="K24" s="126" t="s">
+        <v>17</v>
+      </c>
+      <c r="L24" s="126"/>
       <c r="M24" s="77" t="s">
         <v>39</v>
       </c>
@@ -4361,13 +4364,13 @@
       <c r="F37" s="59"/>
       <c r="G37" s="59"/>
       <c r="H37" s="58"/>
-      <c r="I37" s="119" t="s">
+      <c r="I37" s="118" t="s">
         <v>38</v>
       </c>
-      <c r="J37" s="118"/>
-      <c r="K37" s="118"/>
-      <c r="L37" s="118"/>
-      <c r="M37" s="118"/>
+      <c r="J37" s="117"/>
+      <c r="K37" s="117"/>
+      <c r="L37" s="117"/>
+      <c r="M37" s="117"/>
       <c r="N37" s="47"/>
     </row>
     <row r="38" spans="1:14" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -4427,7 +4430,7 @@
     </row>
     <row r="41" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="45"/>
-      <c r="B41" s="146" t="s">
+      <c r="B41" s="145" t="s">
         <v>35</v>
       </c>
       <c r="C41" s="56"/>
@@ -4446,7 +4449,7 @@
       <c r="N41" s="47"/>
     </row>
     <row r="42" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="149"/>
+      <c r="B42" s="148"/>
       <c r="C42" s="56"/>
       <c r="D42" s="56"/>
       <c r="E42" s="56"/>
@@ -4460,7 +4463,7 @@
       <c r="N42" s="47"/>
     </row>
     <row r="43" spans="1:14" ht="18.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="149"/>
+      <c r="B43" s="148"/>
       <c r="C43" s="56"/>
       <c r="D43" s="56"/>
       <c r="E43" s="56"/>
@@ -4475,7 +4478,7 @@
       <c r="N43" s="47"/>
     </row>
     <row r="44" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="149"/>
+      <c r="B44" s="148"/>
       <c r="C44" s="56"/>
       <c r="D44" s="56"/>
       <c r="E44" s="56"/>
@@ -4490,19 +4493,19 @@
       <c r="N44" s="47"/>
     </row>
     <row r="45" spans="1:14" s="52" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="145"/>
-      <c r="B45" s="147"/>
+      <c r="A45" s="144"/>
+      <c r="B45" s="146"/>
       <c r="C45" s="55"/>
       <c r="D45" s="55"/>
       <c r="E45" s="55"/>
       <c r="F45" s="54"/>
       <c r="G45" s="54"/>
       <c r="H45" s="53"/>
-      <c r="I45" s="120"/>
-      <c r="J45" s="148"/>
-      <c r="K45" s="121"/>
-      <c r="L45" s="121"/>
-      <c r="M45" s="121"/>
+      <c r="I45" s="119"/>
+      <c r="J45" s="147"/>
+      <c r="K45" s="120"/>
+      <c r="L45" s="120"/>
+      <c r="M45" s="120"/>
       <c r="N45" s="78"/>
     </row>
     <row r="46" spans="1:14" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4519,6 +4522,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="70" fitToHeight="2" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="68" fitToHeight="2" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>